<commit_message>
Batch 16 shipped: wave 1, leftovers, JIC tees, 2404, 5405, corner-puck fix
User 2026-10-19: "Yes, ship batch 16 as planned." 25 masters went into 11_MASTERS (not in git):
9 new (0304 0306 1502 2504 2505 2606 2609 2611 2404) and 16 replaced. This commit carries
the rest: 24 macros + 25 reports (03_SCRIPTS), 24 SW2 + 12 review tables (04_DESIGN_TABLES),
the puck-fix toolchain in tools/ (PUCK_INSET 0.0005 in gen_tee.py), QA_Log #170-#172 and
Topologies notes, coverage refresh, RUN_ME_batch16.txt, PROJECT_STATUS / CLAUDE.md /
NEXT_SESSION_PROMPT_2026-10-18 updates, and the ship evidence (tools/_out/ship_20261019:
plan, checks, scripts; puckfix_20261009 dry-run verdict). 1,103 of 1,804 configurations
in a master. Regenerate elbow roots and the 12 changed tables from this state.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/00_DOCS/OMi_Coverage_2026-09-24.xlsx
+++ b/00_DOCS/OMi_Coverage_2026-09-24.xlsx
@@ -446,7 +446,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>OMi carbon-steel library - coverage by OMi part number, enumerated 2026-10-08 from the OMi feed extract, every design table and 11_MASTERS</t>
+          <t>OMi carbon-steel library - coverage by OMi part number, enumerated 2026-10-19 from the OMi feed extract, every design table and 11_MASTERS</t>
         </is>
       </c>
     </row>
@@ -484,7 +484,7 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>943</v>
+        <v>1050</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>98</v>
+        <v>50</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
@@ -604,7 +604,7 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
@@ -704,7 +704,7 @@
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>232</v>
+        <v>208</v>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
@@ -764,7 +764,7 @@
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>266</v>
+        <v>236</v>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
@@ -824,7 +824,7 @@
         </is>
       </c>
       <c r="C21" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
@@ -955,7 +955,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1045,42 +1045,42 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Needs one specific item (see note)</t>
+          <t>adjustable ORB stud (nut/washer) sizes + a new module</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>fold into the base master (your yes, 2026-09-25) - needs one Brennan STEP to see where the extra length goes</t>
+          <t>adjustable ORB stud + locknut (4601)</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>STEP</t>
+          <t>6801-XX-XX-NWO-FG per ORB size</t>
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>2404-L-04-04 2404-L-06-04 2404-L-06-06 2404-L-08-08 2404-L-12-12 6400-L-04-04-O 6400-L-06-06-O 6400-L-08-08-O 6400-L-10-10-O 6400-L-12-12-O 6400-L-16-16-O</t>
+          <t>4601-06-06-NWO-FG 4601-08-08-NWO-FG 4601-10-10-NWO-FG 4601-12-12-NWO-FG 4601-16-12-NWO-FG 4601-32-32-NWO-FG</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>adjustable ORB stud (nut/washer) sizes + a new module</t>
+          <t>Needs one specific item (see note)</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>adjustable ORB stud + locknut (4601)</t>
+          <t>fold into the base master (your yes, 2026-09-25) - needs one Brennan STEP to see where the extra length goes</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>6801-XX-XX-NWO-FG per ORB size</t>
+          <t>STEP</t>
         </is>
       </c>
       <c r="D5" s="3" t="n">
@@ -1088,7 +1088,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>4601-06-06-NWO-FG 4601-08-08-NWO-FG 4601-10-10-NWO-FG 4601-12-12-NWO-FG 4601-16-12-NWO-FG 4601-32-32-NWO-FG</t>
+          <t>6400-L-04-04-O 6400-L-06-06-O 6400-L-08-08-O 6400-L-10-10-O 6400-L-12-12-O 6400-L-16-16-O</t>
         </is>
       </c>
     </row>
@@ -1175,12 +1175,12 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>NPSM swivel -02</t>
+          <t>NPSM swivel -16</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>1404-02-02</t>
+          <t>1404-16-16</t>
         </is>
       </c>
       <c r="D9" s="3" t="n">
@@ -1188,24 +1188,24 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>1501-04-02-FG 1502-02-02-FG 1503-02-02-FG</t>
+          <t>1503-12-16-FG 1503-16-16-FG 1503-20-16-FG</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>female NPSM swivel size</t>
+          <t>Needs one specific item (see note)</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>NPSM swivel -16</t>
+          <t>fixed ORB -14 groove unmeasured</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>1404-16-16</t>
+          <t>6400-14-14-O</t>
         </is>
       </c>
       <c r="D10" s="3" t="n">
@@ -1213,24 +1213,24 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>1503-12-16-FG 1503-16-16-FG 1503-20-16-FG</t>
+          <t>6400-12-14-O 6400-14-14-O 6400-16-14-O</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Needs one specific item (see note)</t>
+          <t>adjustable ORB stud (nut/washer) sizes + a new module</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>fixed ORB -14 groove unmeasured</t>
+          <t>adjustable ORB stud + locknut (6801LL)</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>6400-14-14-O</t>
+          <t>6801-XX-XX-NWO-FG per ORB size</t>
         </is>
       </c>
       <c r="D11" s="3" t="n">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>6400-12-14-O 6400-14-14-O 6400-16-14-O</t>
+          <t>6801-LL-04-04-NWO-FG 6801-LL-06-06-NWO-FG 6801-LL-08-08-NWO-FG</t>
         </is>
       </c>
     </row>
@@ -1250,7 +1250,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>adjustable ORB stud + locknut (6801LL)</t>
+          <t>adjustable ORB stud + locknut (6805)</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>6801-LL-04-04-NWO-FG 6801-LL-06-06-NWO-FG 6801-LL-08-08-NWO-FG</t>
+          <t>6805-06-04-NWO-FG 6805-08-06-NWO-FG 6805-12-12-NWO-FG</t>
         </is>
       </c>
     </row>
@@ -1275,7 +1275,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>adjustable ORB stud + locknut (6805)</t>
+          <t>adjustable ORB stud + locknut (6901)</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -1288,32 +1288,32 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>6805-06-04-NWO-FG 6805-08-06-NWO-FG 6805-12-12-NWO-FG</t>
+          <t>6901-06-04-NWO-FG 6901-06-06-NWO-FG 6901-10-08-NWO-FG</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>adjustable ORB stud (nut/washer) sizes + a new module</t>
+          <t>Needs one specific item (see note)</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>adjustable ORB stud + locknut (6901)</t>
+          <t>OMi-filled 2026-10-02 (was BUILD-MISSING</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>6801-XX-XX-NWO-FG per ORB size</t>
+          <t>TFA</t>
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>6901-06-04-NWO-FG 6901-06-06-NWO-FG 6901-10-08-NWO-FG</t>
+          <t>0304-C-02 0306-02</t>
         </is>
       </c>
     </row>
@@ -1325,12 +1325,12 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>NPSM swivel -24</t>
+          <t>NPSM swivel -02</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>1404-24-24</t>
+          <t>1404-02-02</t>
         </is>
       </c>
       <c r="D15" s="3" t="n">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>1501-24-24-FG 1503-24-24-FG</t>
+          <t>1501-04-02-FG 1503-02-02-FG</t>
         </is>
       </c>
     </row>
@@ -1350,12 +1350,12 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>NPSM swivel -04</t>
+          <t>NPSM swivel -24</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>1404-04-04</t>
+          <t>1404-24-24</t>
         </is>
       </c>
       <c r="D16" s="3" t="n">
@@ -1363,7 +1363,7 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>1502-04-04-FG 1503-04-04-FG</t>
+          <t>1501-24-24-FG 1503-24-24-FG</t>
         </is>
       </c>
     </row>
@@ -1375,12 +1375,12 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>NPSM swivel -06</t>
+          <t>NPSM swivel -04</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>1404-06-06</t>
+          <t>1404-04-04</t>
         </is>
       </c>
       <c r="D17" s="3" t="n">
@@ -1388,7 +1388,7 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>1503-06-06-FG 1503-08-06-FG</t>
+          <t>1502-04-04-FG 1503-04-04-FG</t>
         </is>
       </c>
     </row>
@@ -1400,12 +1400,12 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>NPSM swivel -12</t>
+          <t>NPSM swivel -06</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>1404-12-12</t>
+          <t>1404-06-06</t>
         </is>
       </c>
       <c r="D18" s="3" t="n">
@@ -1413,32 +1413,32 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>1503-12-12-FG 1503-16-12-FG</t>
+          <t>1503-06-06-FG 1503-08-06-FG</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Needs one specific item (see note)</t>
+          <t>female NPSM swivel size</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>body checked on the Brennan 1503-08-08-FG STEP - needs a pipe-thread helper for the 45 deg leg (my work)</t>
+          <t>NPSM swivel -12</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>1503-08-08-FG</t>
+          <t>1404-12-12</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>1503-08-08-FG</t>
+          <t>1503-12-12-FG 1503-16-12-FG</t>
         </is>
       </c>
     </row>
@@ -1450,12 +1450,12 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>the body corner would stick out beside the swivel neck at this size - needs a Brennan 1503-12-08-FG STEP</t>
+          <t>body checked on the Brennan 1503-08-08-FG STEP - needs a pipe-thread helper for the 45 deg leg (my work)</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>1503-12-08-FG</t>
+          <t>1503-08-08-FG</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
@@ -1463,24 +1463,24 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>1503-12-08-FG</t>
+          <t>1503-08-08-FG</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>female NPSM swivel size</t>
+          <t>Needs one specific item (see note)</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>NPSM swivel -20</t>
+          <t>the body corner would stick out beside the swivel neck at this size - needs a Brennan 1503-12-08-FG STEP</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>1404-20-20</t>
+          <t>1503-12-08-FG</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
@@ -1488,7 +1488,7 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>1503-20-20-FG</t>
+          <t>1503-12-08-FG</t>
         </is>
       </c>
     </row>
@@ -1500,12 +1500,12 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>NPSM swivel -32</t>
+          <t>NPSM swivel -20</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>1404-32-32</t>
+          <t>1404-20-20</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
@@ -1513,24 +1513,24 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>1503-32-32-FG</t>
+          <t>1503-20-20-FG</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>female JIC port size</t>
+          <t>female NPSM swivel size</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>female JIC -16</t>
+          <t>NPSM swivel -32</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>2406-16-xx</t>
+          <t>1404-32-32</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -1538,24 +1538,24 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>2406-16-04</t>
+          <t>1503-32-32-FG</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>female ORB port size</t>
+          <t>female JIC port size</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>female ORB -20 port</t>
+          <t>female JIC -16</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>6404/6410</t>
+          <t>2406-16-xx</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>6410-32-20-O</t>
+          <t>2406-16-04</t>
         </is>
       </c>
     </row>
@@ -1575,7 +1575,7 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>female ORB -24 port</t>
+          <t>female ORB -20 port</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
@@ -1588,24 +1588,24 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>6410-32-24-O</t>
+          <t>6410-32-20-O</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>adjustable ORB stud (nut/washer) sizes + a new module</t>
+          <t>female ORB port size</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>adjustable ORB stud + locknut (6802)</t>
+          <t>female ORB -24 port</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>6801-XX-XX-NWO-FG per ORB size</t>
+          <t>6404/6410</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1613,7 +1613,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>6802-04-06-NWO-FG</t>
+          <t>6410-32-24-O</t>
         </is>
       </c>
     </row>
@@ -1625,7 +1625,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>adjustable ORB stud + locknut (6806)</t>
+          <t>adjustable ORB stud + locknut (6802)</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -1638,7 +1638,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>6806-04-04-NWO-FG</t>
+          <t>6802-04-06-NWO-FG</t>
         </is>
       </c>
     </row>
@@ -1650,7 +1650,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>adjustable ORB stud + locknut (6807)</t>
+          <t>adjustable ORB stud + locknut (6806)</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -1663,7 +1663,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>6807-06-06-NWO-FG</t>
+          <t>6806-04-04-NWO-FG</t>
         </is>
       </c>
     </row>
@@ -1675,7 +1675,7 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>adjustable ORB stud + locknut (6902)</t>
+          <t>adjustable ORB stud + locknut (6807)</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
@@ -1687,6 +1687,31 @@
         <v>1</v>
       </c>
       <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>6807-06-06-NWO-FG</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>adjustable ORB stud (nut/washer) sizes + a new module</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>adjustable ORB stud + locknut (6902)</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>6801-XX-XX-NWO-FG per ORB size</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
         <is>
           <t>6902-12-12-NWO-FG</t>
         </is>
@@ -1750,11 +1775,11 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>232</v>
+        <v>208</v>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>1501-16-20-FG 1501-20-16-FG 1502-06-06-FG 1502-08-08-FG 1502-12-12-FG 1502-16-16-FG 1502-20-20-FG 1502-24-24-FG 1502-32-32-FG 1503-04-02-FG 1503-04-06-FG 1503-06-04-FG 1503-06-08-FG 1503-08-12-FG 1504-06-06-FG 1504-24-24-FG 1601-02-02-02-FG 1601-04-04-04-FG 1601-06-06-06-FG 1601-08-08-08-FG 1601-12-12-12-FG 1601-16-16-16-FG 1602-06-06-06-FG 1602-08-08-08-FG 1602-12-12-12-FG 1603-02-02-02-FG 1603-04-04-04-FG 1603-06-06-06-FG 1603-08-08-08-FG 1603-12-12-12-FG 1603-16-16-16-FG 1703-24-24-FG 1704-24-24-FG 1704-32-32-FG 2500-06-04-FG 2500-08-06-FG 2500-12-08-FG 2500-12-10-FG 2501-LL-04-02-FG 2501-LL-04-04-FG 2501-LL-06-04-FG 2501-LL-06-06-FG 2501-LL-08-08-FG 2501-LL-12-12-FG 2501-LL-16-16-FG 2502-06-08-FG 2502-08-04-FG 2502-12-08-FG 2502-16-20-FG 2502-24-24-FG 2504-04-04-FG 2504-06-06-FG 2504-08-08-FG 2504-12-12-FG 2505-08-08-FG 2505-12-12-FG 2505-16-16-FG 2602-08-08-08-FG 2606-04-04-04-FG 2606-06-06-06-FG 2606-08-08-08-FG 2606-16-16-16-FG 2611-06-06-06-FG 2611-12-12-12-FG 4501-06-04-FG 4501-06-06-FG 4501-08-06-FG 4501-08-08-FG 4501-08-12-FG 4501-10-08-FG 4501-12-08-FG 4501-12-12-FG 4501-16-12-FG 4501-16-16-FG 4501-20-20-FG 4503-04-04-FG 4503-08-08-FG 4503-12-12-FG 4503-16-12-FG 4503-16-16-FG 4503-20-20-FG 4503-24-24-FG 4601-04-04-NWO-FG 4601-08-06-NWO-FG 4601-12-10-NWO-FG 4601-16-16-NWO-FG 4601-16-20-NWO-FG 4601-20-16-NWO-FG 4601-20-20-NWO-FG 4601-24-20-NWO-FG 4601-24-24-NWO-FG 4603-16-16-NWO-FG 5501-02-02-FG 5501-04-04-FG 5501-06-06-FG 5501-08-08-FG 5501-12-12-FG 5501-16-16-FG 5501-20-20-FG 5502-02-04-FG 5502-06-08-FG 5502-12-08-FG 5502-20-16-FG 5503-16-16-FG 5503-20-20-FG 5503-24-24-FG 5503-32-32-FG 5504-06-04-FG 5504-06-06-FG 5504-08-06-FG 5504-20-20-FG 5504-24-24-FG 5504-32-32-FG 5505-02-02-FG 5505-06-06-FG 5505-08-08-FG 5505-12-12-FG 5505-16-16-FG 5601-04-04-04-FG 5601-06-06-06-FG 5602-02-02-02-FG 5602-06-06-06-FG 5602-12-12-12-FG 5602-16-16-16-FG 5602-20-20-20-FG 5602-24-24-24-FG 5602-32-32-32-FG 5603-04-04-04-FG 5603-06-06-06-FG 5603-08-08-08-FG 5603-16-16-16-FG 5603-20-20-20-FG 5604-02-02-02-FG 5604-12-12-12-FG 5604-16-16-16-FG 5604-20-20-20-FG 5605-02-02-02-FG 5605-12-12-12-FG 5605-16-16-16-FG 5605-20-20-20-FG 5605-32-32-32-FG 5652-02-02-02-02-FG 5652-04-04-04-04-FG 5652-06-06-06-06-FG 5652-08-08-08-08-FG 5652-12-12-12-12-FG 5652-16-16-16-16-FG 5652-20-20-20-20-FG 5652-24-24-24-24-FG 6500-04-06-FG 6500-12-08-FG 6500-12-16-FG 6500-16-12-FG 6500-L-04-04-FG 6500-L-06-06-FG 6500-L-08-08-FG 6500-L-12-12-FG 6500-L-16-16-FG 6501-06-06-FG 6501-12-12-FG 6503-04-04-FG 6503-06-06-FG 6503-12-12-FG 6503-16-16-FG 6603-06-06-06-FG 6603-16-16-16-FG 6606-06-06-06-FG 6606-12-12-12-FG 6801-08-04-NWO-FG 6801-08-16-NWO-FG 6801-12-20-NWO-FG 6801-16-24-NWO-FG 6801-24-16-NWO-FG 6801-L-16-16-NWO-FG 6801-L-20-20-NWO-FG 6801-LL-12-12-NWO-FG 6801-LL-16-16-NWO-FG 6801-LL-20-20-NWO-FG 6802-06-10-NWO-FG 6802-08-12-NWO-FG 6803-08-08-06-NWO-FG 6803-08-08-10-NWO-FG 6803-24-24-24-NWO-FG 6804-24-24-24-NWO-FG 6805-04-02-NWO-FG 6805-04-04-NWO-FG 6805-06-06-NWO-FG 6805-08-08-NWO-FG 6805-10-08-NWO-FG 6805-12-08-NWO-FG 6805-16-12-NWO-FG 6805-16-16-NWO-FG 6805-20-20-NWO-FG 6806-06-04-NWO-FG 6806-06-06-NWO-FG 6806-08-06-NWO-FG 6806-08-08-NWO-FG 6806-10-08-NWO-FG 6806-12-12-NWO-FG 6806-16-16-NWO-FG 6806-20-20-NWO-FG 6806-24-24-NWO-FG 6807-04-04-NWO-FG 6807-08-06-NWO-FG 6807-08-08-NWO-FG 6807-12-12-NWO-FG 6809-10-10-NWO-FG 6809-12-12-NWO-FG 6809-16-16-NWO-FG 6809-20-20-NWO-FG 6810-12-12-NWO-FG 6901-04-04-NWO-FG 6901-04-06-NWO-FG 6901-06-08-NWO-FG 6901-10-12-NWO-FG 6901-12-06-NWO-FG 6901-12-08-NWO-FG 6901-12-12-NWO-FG 6901-12-16-NWO-FG 6901-16-12-NWO-FG 6901-16-16-NWO-FG 6901-20-16-NWO-FG 6901-20-20-NWO-FG 6901-24-24-NWO-FG 6902-04-04-NWO-FG 6902-06-04-NWO-FG 6902-06-06-NWO-FG 6902-08-06-NWO-FG 6902-08-08-NWO-FG 6902-10-08-NWO-FG 6902-10-12-NWO-FG 6902-16-16-NWO-FG</t>
+          <t>1501-16-20-FG 1501-20-16-FG 1502-06-06-FG 1502-08-08-FG 1502-12-12-FG 1502-16-16-FG 1502-20-20-FG 1502-24-24-FG 1502-32-32-FG 1503-04-02-FG 1503-04-06-FG 1503-06-04-FG 1503-06-08-FG 1503-08-12-FG 1504-06-06-FG 1504-24-24-FG 1601-02-02-02-FG 1601-04-04-04-FG 1601-06-06-06-FG 1601-08-08-08-FG 1601-12-12-12-FG 1601-16-16-16-FG 1602-06-06-06-FG 1602-08-08-08-FG 1602-12-12-12-FG 1603-02-02-02-FG 1603-04-04-04-FG 1603-06-06-06-FG 1603-08-08-08-FG 1603-12-12-12-FG 1603-16-16-16-FG 1703-24-24-FG 1704-24-24-FG 1704-32-32-FG 2500-06-04-FG 2500-08-06-FG 2500-12-08-FG 2500-12-10-FG 2501-LL-04-02-FG 2501-LL-04-04-FG 2501-LL-06-04-FG 2501-LL-06-06-FG 2501-LL-08-08-FG 2501-LL-12-12-FG 2501-LL-16-16-FG 2502-06-08-FG 2502-08-04-FG 2502-12-08-FG 2502-16-20-FG 2502-24-24-FG 2602-08-08-08-FG 4501-06-04-FG 4501-06-06-FG 4501-08-06-FG 4501-08-08-FG 4501-08-12-FG 4501-10-08-FG 4501-12-08-FG 4501-12-12-FG 4501-16-12-FG 4501-16-16-FG 4501-20-20-FG 4503-04-04-FG 4503-08-08-FG 4503-12-12-FG 4503-16-12-FG 4503-16-16-FG 4503-20-20-FG 4503-24-24-FG 4601-04-04-NWO-FG 4601-08-06-NWO-FG 4601-12-10-NWO-FG 4601-16-16-NWO-FG 4601-16-20-NWO-FG 4601-20-16-NWO-FG 4601-20-20-NWO-FG 4601-24-20-NWO-FG 4601-24-24-NWO-FG 4603-16-16-NWO-FG 5501-02-02-FG 5501-04-04-FG 5501-06-06-FG 5501-08-08-FG 5501-12-12-FG 5501-16-16-FG 5501-20-20-FG 5502-02-04-FG 5502-06-08-FG 5502-12-08-FG 5502-20-16-FG 5503-16-16-FG 5503-20-20-FG 5503-24-24-FG 5503-32-32-FG 5504-06-04-FG 5504-06-06-FG 5504-08-06-FG 5504-20-20-FG 5504-24-24-FG 5504-32-32-FG 5505-02-02-FG 5505-06-06-FG 5505-08-08-FG 5505-12-12-FG 5505-16-16-FG 5601-04-04-04-FG 5601-06-06-06-FG 5602-02-02-02-FG 5602-06-06-06-FG 5602-12-12-12-FG 5602-16-16-16-FG 5602-20-20-20-FG 5602-24-24-24-FG 5602-32-32-32-FG 5603-04-04-04-FG 5603-06-06-06-FG 5603-08-08-08-FG 5603-16-16-16-FG 5603-20-20-20-FG 5604-02-02-02-FG 5604-12-12-12-FG 5604-16-16-16-FG 5604-20-20-20-FG 5605-02-02-02-FG 5605-12-12-12-FG 5605-16-16-16-FG 5605-20-20-20-FG 5605-32-32-32-FG 5652-02-02-02-02-FG 5652-04-04-04-04-FG 5652-06-06-06-06-FG 5652-08-08-08-08-FG 5652-12-12-12-12-FG 5652-16-16-16-16-FG 5652-20-20-20-20-FG 5652-24-24-24-24-FG 6503-04-04-FG 6503-06-06-FG 6503-12-12-FG 6503-16-16-FG 6603-06-06-06-FG 6603-16-16-16-FG 6606-06-06-06-FG 6606-12-12-12-FG 6801-08-04-NWO-FG 6801-08-16-NWO-FG 6801-12-20-NWO-FG 6801-16-24-NWO-FG 6801-24-16-NWO-FG 6801-L-16-16-NWO-FG 6801-L-20-20-NWO-FG 6801-LL-12-12-NWO-FG 6801-LL-16-16-NWO-FG 6801-LL-20-20-NWO-FG 6802-06-10-NWO-FG 6802-08-12-NWO-FG 6803-08-08-06-NWO-FG 6803-08-08-10-NWO-FG 6803-24-24-24-NWO-FG 6804-24-24-24-NWO-FG 6805-04-02-NWO-FG 6805-04-04-NWO-FG 6805-06-06-NWO-FG 6805-08-08-NWO-FG 6805-10-08-NWO-FG 6805-12-08-NWO-FG 6805-16-12-NWO-FG 6805-16-16-NWO-FG 6805-20-20-NWO-FG 6806-06-04-NWO-FG 6806-06-06-NWO-FG 6806-08-06-NWO-FG 6806-08-08-NWO-FG 6806-10-08-NWO-FG 6806-12-12-NWO-FG 6806-16-16-NWO-FG 6806-20-20-NWO-FG 6806-24-24-NWO-FG 6807-04-04-NWO-FG 6807-08-06-NWO-FG 6807-08-08-NWO-FG 6807-12-12-NWO-FG 6809-10-10-NWO-FG 6809-12-12-NWO-FG 6809-16-16-NWO-FG 6809-20-20-NWO-FG 6810-12-12-NWO-FG 6901-04-04-NWO-FG 6901-04-06-NWO-FG 6901-06-08-NWO-FG 6901-10-12-NWO-FG 6901-12-06-NWO-FG 6901-12-08-NWO-FG 6901-12-12-NWO-FG 6901-12-16-NWO-FG 6901-16-12-NWO-FG 6901-16-16-NWO-FG 6901-20-16-NWO-FG 6901-20-20-NWO-FG 6901-24-24-NWO-FG 6902-04-04-NWO-FG 6902-06-04-NWO-FG 6902-06-06-NWO-FG 6902-08-06-NWO-FG 6902-08-08-NWO-FG 6902-10-08-NWO-FG 6902-10-12-NWO-FG 6902-16-16-NWO-FG</t>
         </is>
       </c>
     </row>
@@ -1769,7 +1794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U135"/>
+  <dimension ref="A1:U134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1908,7 +1933,9 @@
           <t>0304</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n"/>
+      <c r="B2" s="3" t="n">
+        <v>12</v>
+      </c>
       <c r="C2" s="3" t="n"/>
       <c r="D2" s="3" t="n"/>
       <c r="E2" s="3" t="n"/>
@@ -1919,12 +1946,12 @@
       <c r="J2" s="3" t="n"/>
       <c r="K2" s="3" t="n"/>
       <c r="L2" s="3" t="n"/>
-      <c r="M2" s="3" t="n"/>
+      <c r="M2" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="N2" s="3" t="n"/>
       <c r="O2" s="3" t="n"/>
-      <c r="P2" s="3" t="n">
-        <v>13</v>
-      </c>
+      <c r="P2" s="3" t="n"/>
       <c r="Q2" s="3" t="n"/>
       <c r="R2" s="3" t="n"/>
       <c r="S2" s="3" t="n"/>
@@ -1939,7 +1966,9 @@
           <t>0306</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n"/>
+      <c r="B3" s="3" t="n">
+        <v>11</v>
+      </c>
       <c r="C3" s="3" t="n"/>
       <c r="D3" s="3" t="n"/>
       <c r="E3" s="3" t="n"/>
@@ -1950,12 +1979,12 @@
       <c r="J3" s="3" t="n"/>
       <c r="K3" s="3" t="n"/>
       <c r="L3" s="3" t="n"/>
-      <c r="M3" s="3" t="n"/>
+      <c r="M3" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="N3" s="3" t="n"/>
       <c r="O3" s="3" t="n"/>
-      <c r="P3" s="3" t="n">
-        <v>12</v>
-      </c>
+      <c r="P3" s="3" t="n"/>
       <c r="Q3" s="3" t="n"/>
       <c r="R3" s="3" t="n"/>
       <c r="S3" s="3" t="n"/>
@@ -2224,14 +2253,16 @@
           <t>1502</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="C12" s="3" t="n"/>
       <c r="D12" s="3" t="n"/>
       <c r="E12" s="3" t="n"/>
       <c r="F12" s="3" t="n"/>
       <c r="G12" s="3" t="n"/>
       <c r="H12" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I12" s="3" t="n"/>
       <c r="J12" s="3" t="n"/>
@@ -2868,10 +2899,10 @@
           <t>2404</t>
         </is>
       </c>
-      <c r="B32" s="3" t="n"/>
-      <c r="C32" s="3" t="n">
-        <v>48</v>
-      </c>
+      <c r="B32" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="C32" s="3" t="n"/>
       <c r="D32" s="3" t="n"/>
       <c r="E32" s="3" t="n"/>
       <c r="F32" s="3" t="n"/>
@@ -2890,7 +2921,7 @@
       <c r="S32" s="3" t="n"/>
       <c r="T32" s="3" t="n"/>
       <c r="U32" s="3" t="n">
-        <v>48</v>
+        <v>57</v>
       </c>
     </row>
     <row r="33">
@@ -2910,9 +2941,7 @@
       <c r="J33" s="3" t="n"/>
       <c r="K33" s="3" t="n"/>
       <c r="L33" s="3" t="n"/>
-      <c r="M33" s="3" t="n">
-        <v>5</v>
-      </c>
+      <c r="M33" s="3" t="n"/>
       <c r="N33" s="3" t="n"/>
       <c r="O33" s="3" t="n"/>
       <c r="P33" s="3" t="n">
@@ -2923,7 +2952,7 @@
       <c r="S33" s="3" t="n"/>
       <c r="T33" s="3" t="n"/>
       <c r="U33" s="3" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -2944,7 +2973,7 @@
       <c r="K34" s="3" t="n"/>
       <c r="L34" s="3" t="n"/>
       <c r="M34" s="3" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="N34" s="3" t="n"/>
       <c r="O34" s="3" t="n"/>
@@ -2954,7 +2983,7 @@
       <c r="S34" s="3" t="n"/>
       <c r="T34" s="3" t="n"/>
       <c r="U34" s="3" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35">
@@ -3285,7 +3314,9 @@
           <t>2504</t>
         </is>
       </c>
-      <c r="B45" s="3" t="n"/>
+      <c r="B45" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="C45" s="3" t="n"/>
       <c r="D45" s="3" t="n"/>
       <c r="E45" s="3" t="n"/>
@@ -3298,9 +3329,7 @@
       <c r="L45" s="3" t="n"/>
       <c r="M45" s="3" t="n"/>
       <c r="N45" s="3" t="n"/>
-      <c r="O45" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="O45" s="3" t="n"/>
       <c r="P45" s="3" t="n"/>
       <c r="Q45" s="3" t="n"/>
       <c r="R45" s="3" t="n"/>
@@ -3316,7 +3345,9 @@
           <t>2505</t>
         </is>
       </c>
-      <c r="B46" s="3" t="n"/>
+      <c r="B46" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="C46" s="3" t="n"/>
       <c r="D46" s="3" t="n"/>
       <c r="E46" s="3" t="n"/>
@@ -3327,11 +3358,11 @@
       <c r="J46" s="3" t="n"/>
       <c r="K46" s="3" t="n"/>
       <c r="L46" s="3" t="n"/>
-      <c r="M46" s="3" t="n"/>
+      <c r="M46" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="N46" s="3" t="n"/>
-      <c r="O46" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="O46" s="3" t="n"/>
       <c r="P46" s="3" t="n"/>
       <c r="Q46" s="3" t="n"/>
       <c r="R46" s="3" t="n"/>
@@ -3504,7 +3535,9 @@
           <t>2606</t>
         </is>
       </c>
-      <c r="B52" s="3" t="n"/>
+      <c r="B52" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="C52" s="3" t="n"/>
       <c r="D52" s="3" t="n"/>
       <c r="E52" s="3" t="n"/>
@@ -3517,12 +3550,8 @@
       <c r="L52" s="3" t="n"/>
       <c r="M52" s="3" t="n"/>
       <c r="N52" s="3" t="n"/>
-      <c r="O52" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="P52" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="O52" s="3" t="n"/>
+      <c r="P52" s="3" t="n"/>
       <c r="Q52" s="3" t="n"/>
       <c r="R52" s="3" t="n"/>
       <c r="S52" s="3" t="n"/>
@@ -3537,7 +3566,9 @@
           <t>2609</t>
         </is>
       </c>
-      <c r="B53" s="3" t="n"/>
+      <c r="B53" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="C53" s="3" t="n"/>
       <c r="D53" s="3" t="n"/>
       <c r="E53" s="3" t="n"/>
@@ -3551,9 +3582,7 @@
       <c r="M53" s="3" t="n"/>
       <c r="N53" s="3" t="n"/>
       <c r="O53" s="3" t="n"/>
-      <c r="P53" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="P53" s="3" t="n"/>
       <c r="Q53" s="3" t="n"/>
       <c r="R53" s="3" t="n"/>
       <c r="S53" s="3" t="n"/>
@@ -3568,7 +3597,9 @@
           <t>2611</t>
         </is>
       </c>
-      <c r="B54" s="3" t="n"/>
+      <c r="B54" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="C54" s="3" t="n"/>
       <c r="D54" s="3" t="n"/>
       <c r="E54" s="3" t="n"/>
@@ -3581,15 +3612,13 @@
       <c r="L54" s="3" t="n"/>
       <c r="M54" s="3" t="n"/>
       <c r="N54" s="3" t="n"/>
-      <c r="O54" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="P54" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="O54" s="3" t="n"/>
+      <c r="P54" s="3" t="n"/>
       <c r="Q54" s="3" t="n"/>
       <c r="R54" s="3" t="n"/>
-      <c r="S54" s="3" t="n"/>
+      <c r="S54" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="T54" s="3" t="n"/>
       <c r="U54" s="3" t="n">
         <v>3</v>
@@ -5197,7 +5226,7 @@
         </is>
       </c>
       <c r="B104" s="3" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="C104" s="3" t="n"/>
       <c r="D104" s="3" t="n"/>
@@ -5211,9 +5240,7 @@
       <c r="L104" s="3" t="n"/>
       <c r="M104" s="3" t="n"/>
       <c r="N104" s="3" t="n"/>
-      <c r="O104" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="O104" s="3" t="n"/>
       <c r="P104" s="3" t="n">
         <v>4</v>
       </c>
@@ -5222,16 +5249,18 @@
       <c r="S104" s="3" t="n"/>
       <c r="T104" s="3" t="n"/>
       <c r="U104" s="3" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
         <is>
-          <t>6500L</t>
-        </is>
-      </c>
-      <c r="B105" s="3" t="n"/>
+          <t>6501</t>
+        </is>
+      </c>
+      <c r="B105" s="3" t="n">
+        <v>14</v>
+      </c>
       <c r="C105" s="3" t="n"/>
       <c r="D105" s="3" t="n"/>
       <c r="E105" s="3" t="n"/>
@@ -5244,22 +5273,22 @@
       <c r="L105" s="3" t="n"/>
       <c r="M105" s="3" t="n"/>
       <c r="N105" s="3" t="n"/>
-      <c r="O105" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="P105" s="3" t="n"/>
+      <c r="O105" s="3" t="n"/>
+      <c r="P105" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="Q105" s="3" t="n"/>
       <c r="R105" s="3" t="n"/>
       <c r="S105" s="3" t="n"/>
       <c r="T105" s="3" t="n"/>
       <c r="U105" s="3" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="3" t="inlineStr">
         <is>
-          <t>6501</t>
+          <t>6502</t>
         </is>
       </c>
       <c r="B106" s="3" t="n">
@@ -5277,11 +5306,9 @@
       <c r="L106" s="3" t="n"/>
       <c r="M106" s="3" t="n"/>
       <c r="N106" s="3" t="n"/>
-      <c r="O106" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="O106" s="3" t="n"/>
       <c r="P106" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q106" s="3" t="n"/>
       <c r="R106" s="3" t="n"/>
@@ -5294,11 +5321,11 @@
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
         <is>
-          <t>6502</t>
+          <t>6503</t>
         </is>
       </c>
       <c r="B107" s="3" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="C107" s="3" t="n"/>
       <c r="D107" s="3" t="n"/>
@@ -5312,26 +5339,26 @@
       <c r="L107" s="3" t="n"/>
       <c r="M107" s="3" t="n"/>
       <c r="N107" s="3" t="n"/>
-      <c r="O107" s="3" t="n"/>
-      <c r="P107" s="3" t="n">
+      <c r="O107" s="3" t="n">
         <v>4</v>
       </c>
+      <c r="P107" s="3" t="n"/>
       <c r="Q107" s="3" t="n"/>
       <c r="R107" s="3" t="n"/>
       <c r="S107" s="3" t="n"/>
       <c r="T107" s="3" t="n"/>
       <c r="U107" s="3" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
         <is>
-          <t>6503</t>
+          <t>6504</t>
         </is>
       </c>
       <c r="B108" s="3" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C108" s="3" t="n"/>
       <c r="D108" s="3" t="n"/>
@@ -5345,26 +5372,26 @@
       <c r="L108" s="3" t="n"/>
       <c r="M108" s="3" t="n"/>
       <c r="N108" s="3" t="n"/>
-      <c r="O108" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="P108" s="3" t="n"/>
+      <c r="O108" s="3" t="n"/>
+      <c r="P108" s="3" t="n">
+        <v>10</v>
+      </c>
       <c r="Q108" s="3" t="n"/>
       <c r="R108" s="3" t="n"/>
       <c r="S108" s="3" t="n"/>
       <c r="T108" s="3" t="n"/>
       <c r="U108" s="3" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
         <is>
-          <t>6504</t>
+          <t>6505</t>
         </is>
       </c>
       <c r="B109" s="3" t="n">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="C109" s="3" t="n"/>
       <c r="D109" s="3" t="n"/>
@@ -5380,7 +5407,7 @@
       <c r="N109" s="3" t="n"/>
       <c r="O109" s="3" t="n"/>
       <c r="P109" s="3" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="Q109" s="3" t="n"/>
       <c r="R109" s="3" t="n"/>
@@ -5393,11 +5420,11 @@
     <row r="110">
       <c r="A110" s="3" t="inlineStr">
         <is>
-          <t>6505</t>
+          <t>6506</t>
         </is>
       </c>
       <c r="B110" s="3" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C110" s="3" t="n"/>
       <c r="D110" s="3" t="n"/>
@@ -5413,24 +5440,26 @@
       <c r="N110" s="3" t="n"/>
       <c r="O110" s="3" t="n"/>
       <c r="P110" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q110" s="3" t="n"/>
       <c r="R110" s="3" t="n"/>
-      <c r="S110" s="3" t="n"/>
+      <c r="S110" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="T110" s="3" t="n"/>
       <c r="U110" s="3" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t>6506</t>
+          <t>6565</t>
         </is>
       </c>
       <c r="B111" s="3" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="C111" s="3" t="n"/>
       <c r="D111" s="3" t="n"/>
@@ -5445,28 +5474,24 @@
       <c r="M111" s="3" t="n"/>
       <c r="N111" s="3" t="n"/>
       <c r="O111" s="3" t="n"/>
-      <c r="P111" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="P111" s="3" t="n"/>
       <c r="Q111" s="3" t="n"/>
-      <c r="R111" s="3" t="n"/>
-      <c r="S111" s="3" t="n">
+      <c r="R111" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="S111" s="3" t="n"/>
       <c r="T111" s="3" t="n"/>
       <c r="U111" s="3" t="n">
-        <v>19</v>
+        <v>9</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="3" t="inlineStr">
         <is>
-          <t>6565</t>
-        </is>
-      </c>
-      <c r="B112" s="3" t="n">
-        <v>8</v>
-      </c>
+          <t>6566</t>
+        </is>
+      </c>
+      <c r="B112" s="3" t="n"/>
       <c r="C112" s="3" t="n"/>
       <c r="D112" s="3" t="n"/>
       <c r="E112" s="3" t="n"/>
@@ -5481,23 +5506,25 @@
       <c r="N112" s="3" t="n"/>
       <c r="O112" s="3" t="n"/>
       <c r="P112" s="3" t="n"/>
-      <c r="Q112" s="3" t="n"/>
-      <c r="R112" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q112" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="R112" s="3" t="n"/>
       <c r="S112" s="3" t="n"/>
       <c r="T112" s="3" t="n"/>
       <c r="U112" s="3" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
         <is>
-          <t>6566</t>
-        </is>
-      </c>
-      <c r="B113" s="3" t="n"/>
+          <t>6600</t>
+        </is>
+      </c>
+      <c r="B113" s="3" t="n">
+        <v>9</v>
+      </c>
       <c r="C113" s="3" t="n"/>
       <c r="D113" s="3" t="n"/>
       <c r="E113" s="3" t="n"/>
@@ -5512,20 +5539,20 @@
       <c r="N113" s="3" t="n"/>
       <c r="O113" s="3" t="n"/>
       <c r="P113" s="3" t="n"/>
-      <c r="Q113" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="R113" s="3" t="n"/>
+      <c r="Q113" s="3" t="n"/>
+      <c r="R113" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="S113" s="3" t="n"/>
       <c r="T113" s="3" t="n"/>
       <c r="U113" s="3" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="3" t="inlineStr">
         <is>
-          <t>6600</t>
+          <t>6602</t>
         </is>
       </c>
       <c r="B114" s="3" t="n">
@@ -5546,24 +5573,20 @@
       <c r="O114" s="3" t="n"/>
       <c r="P114" s="3" t="n"/>
       <c r="Q114" s="3" t="n"/>
-      <c r="R114" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="R114" s="3" t="n"/>
       <c r="S114" s="3" t="n"/>
       <c r="T114" s="3" t="n"/>
       <c r="U114" s="3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
         <is>
-          <t>6602</t>
-        </is>
-      </c>
-      <c r="B115" s="3" t="n">
-        <v>9</v>
-      </c>
+          <t>6603</t>
+        </is>
+      </c>
+      <c r="B115" s="3" t="n"/>
       <c r="C115" s="3" t="n"/>
       <c r="D115" s="3" t="n"/>
       <c r="E115" s="3" t="n"/>
@@ -5576,20 +5599,22 @@
       <c r="L115" s="3" t="n"/>
       <c r="M115" s="3" t="n"/>
       <c r="N115" s="3" t="n"/>
-      <c r="O115" s="3" t="n"/>
+      <c r="O115" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="P115" s="3" t="n"/>
       <c r="Q115" s="3" t="n"/>
       <c r="R115" s="3" t="n"/>
       <c r="S115" s="3" t="n"/>
       <c r="T115" s="3" t="n"/>
       <c r="U115" s="3" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="3" t="inlineStr">
         <is>
-          <t>6603</t>
+          <t>6606</t>
         </is>
       </c>
       <c r="B116" s="3" t="n"/>
@@ -5608,19 +5633,21 @@
       <c r="O116" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="P116" s="3" t="n"/>
+      <c r="P116" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="Q116" s="3" t="n"/>
       <c r="R116" s="3" t="n"/>
       <c r="S116" s="3" t="n"/>
       <c r="T116" s="3" t="n"/>
       <c r="U116" s="3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="3" t="inlineStr">
         <is>
-          <t>6606</t>
+          <t>6701</t>
         </is>
       </c>
       <c r="B117" s="3" t="n"/>
@@ -5636,27 +5663,27 @@
       <c r="L117" s="3" t="n"/>
       <c r="M117" s="3" t="n"/>
       <c r="N117" s="3" t="n"/>
-      <c r="O117" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="P117" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q117" s="3" t="n"/>
+      <c r="O117" s="3" t="n"/>
+      <c r="P117" s="3" t="n"/>
+      <c r="Q117" s="3" t="n">
+        <v>7</v>
+      </c>
       <c r="R117" s="3" t="n"/>
       <c r="S117" s="3" t="n"/>
       <c r="T117" s="3" t="n"/>
       <c r="U117" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="3" t="inlineStr">
         <is>
-          <t>6701</t>
-        </is>
-      </c>
-      <c r="B118" s="3" t="n"/>
+          <t>6801</t>
+        </is>
+      </c>
+      <c r="B118" s="3" t="n">
+        <v>35</v>
+      </c>
       <c r="C118" s="3" t="n"/>
       <c r="D118" s="3" t="n"/>
       <c r="E118" s="3" t="n"/>
@@ -5669,27 +5696,27 @@
       <c r="L118" s="3" t="n"/>
       <c r="M118" s="3" t="n"/>
       <c r="N118" s="3" t="n"/>
-      <c r="O118" s="3" t="n"/>
+      <c r="O118" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="P118" s="3" t="n"/>
-      <c r="Q118" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="R118" s="3" t="n"/>
+      <c r="Q118" s="3" t="n"/>
+      <c r="R118" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="S118" s="3" t="n"/>
       <c r="T118" s="3" t="n"/>
       <c r="U118" s="3" t="n">
-        <v>7</v>
+        <v>41</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="3" t="inlineStr">
         <is>
-          <t>6801</t>
-        </is>
-      </c>
-      <c r="B119" s="3" t="n">
-        <v>35</v>
-      </c>
+          <t>6801L</t>
+        </is>
+      </c>
+      <c r="B119" s="3" t="n"/>
       <c r="C119" s="3" t="n"/>
       <c r="D119" s="3" t="n"/>
       <c r="E119" s="3" t="n"/>
@@ -5699,27 +5726,27 @@
       <c r="I119" s="3" t="n"/>
       <c r="J119" s="3" t="n"/>
       <c r="K119" s="3" t="n"/>
-      <c r="L119" s="3" t="n"/>
+      <c r="L119" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="M119" s="3" t="n"/>
       <c r="N119" s="3" t="n"/>
       <c r="O119" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="P119" s="3" t="n"/>
       <c r="Q119" s="3" t="n"/>
-      <c r="R119" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="R119" s="3" t="n"/>
       <c r="S119" s="3" t="n"/>
       <c r="T119" s="3" t="n"/>
       <c r="U119" s="3" t="n">
-        <v>41</v>
+        <v>6</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="3" t="inlineStr">
         <is>
-          <t>6801L</t>
+          <t>6801LL</t>
         </is>
       </c>
       <c r="B120" s="3" t="n"/>
@@ -5733,12 +5760,12 @@
       <c r="J120" s="3" t="n"/>
       <c r="K120" s="3" t="n"/>
       <c r="L120" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M120" s="3" t="n"/>
       <c r="N120" s="3" t="n"/>
       <c r="O120" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P120" s="3" t="n"/>
       <c r="Q120" s="3" t="n"/>
@@ -5752,10 +5779,12 @@
     <row r="121">
       <c r="A121" s="3" t="inlineStr">
         <is>
-          <t>6801LL</t>
-        </is>
-      </c>
-      <c r="B121" s="3" t="n"/>
+          <t>6802</t>
+        </is>
+      </c>
+      <c r="B121" s="3" t="n">
+        <v>20</v>
+      </c>
       <c r="C121" s="3" t="n"/>
       <c r="D121" s="3" t="n"/>
       <c r="E121" s="3" t="n"/>
@@ -5766,30 +5795,32 @@
       <c r="J121" s="3" t="n"/>
       <c r="K121" s="3" t="n"/>
       <c r="L121" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M121" s="3" t="n"/>
       <c r="N121" s="3" t="n"/>
       <c r="O121" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="P121" s="3" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="P121" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="Q121" s="3" t="n"/>
       <c r="R121" s="3" t="n"/>
       <c r="S121" s="3" t="n"/>
       <c r="T121" s="3" t="n"/>
       <c r="U121" s="3" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>6802</t>
+          <t>6803</t>
         </is>
       </c>
       <c r="B122" s="3" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="C122" s="3" t="n"/>
       <c r="D122" s="3" t="n"/>
@@ -5800,33 +5831,29 @@
       <c r="I122" s="3" t="n"/>
       <c r="J122" s="3" t="n"/>
       <c r="K122" s="3" t="n"/>
-      <c r="L122" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="L122" s="3" t="n"/>
       <c r="M122" s="3" t="n"/>
       <c r="N122" s="3" t="n"/>
       <c r="O122" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="P122" s="3" t="n">
-        <v>1</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="P122" s="3" t="n"/>
       <c r="Q122" s="3" t="n"/>
       <c r="R122" s="3" t="n"/>
       <c r="S122" s="3" t="n"/>
       <c r="T122" s="3" t="n"/>
       <c r="U122" s="3" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="3" t="inlineStr">
         <is>
-          <t>6803</t>
+          <t>6804</t>
         </is>
       </c>
       <c r="B123" s="3" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C123" s="3" t="n"/>
       <c r="D123" s="3" t="n"/>
@@ -5841,7 +5868,7 @@
       <c r="M123" s="3" t="n"/>
       <c r="N123" s="3" t="n"/>
       <c r="O123" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P123" s="3" t="n"/>
       <c r="Q123" s="3" t="n"/>
@@ -5849,18 +5876,16 @@
       <c r="S123" s="3" t="n"/>
       <c r="T123" s="3" t="n"/>
       <c r="U123" s="3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="3" t="inlineStr">
         <is>
-          <t>6804</t>
-        </is>
-      </c>
-      <c r="B124" s="3" t="n">
-        <v>8</v>
-      </c>
+          <t>6805</t>
+        </is>
+      </c>
+      <c r="B124" s="3" t="n"/>
       <c r="C124" s="3" t="n"/>
       <c r="D124" s="3" t="n"/>
       <c r="E124" s="3" t="n"/>
@@ -5870,11 +5895,13 @@
       <c r="I124" s="3" t="n"/>
       <c r="J124" s="3" t="n"/>
       <c r="K124" s="3" t="n"/>
-      <c r="L124" s="3" t="n"/>
+      <c r="L124" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="M124" s="3" t="n"/>
       <c r="N124" s="3" t="n"/>
       <c r="O124" s="3" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="P124" s="3" t="n"/>
       <c r="Q124" s="3" t="n"/>
@@ -5882,13 +5909,13 @@
       <c r="S124" s="3" t="n"/>
       <c r="T124" s="3" t="n"/>
       <c r="U124" s="3" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
         <is>
-          <t>6805</t>
+          <t>6806</t>
         </is>
       </c>
       <c r="B125" s="3" t="n"/>
@@ -5902,26 +5929,28 @@
       <c r="J125" s="3" t="n"/>
       <c r="K125" s="3" t="n"/>
       <c r="L125" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M125" s="3" t="n"/>
       <c r="N125" s="3" t="n"/>
       <c r="O125" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="P125" s="3" t="n"/>
+      <c r="P125" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="Q125" s="3" t="n"/>
       <c r="R125" s="3" t="n"/>
       <c r="S125" s="3" t="n"/>
       <c r="T125" s="3" t="n"/>
       <c r="U125" s="3" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="3" t="inlineStr">
         <is>
-          <t>6806</t>
+          <t>6807</t>
         </is>
       </c>
       <c r="B126" s="3" t="n"/>
@@ -5940,23 +5969,21 @@
       <c r="M126" s="3" t="n"/>
       <c r="N126" s="3" t="n"/>
       <c r="O126" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="P126" s="3" t="n">
-        <v>1</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="P126" s="3" t="n"/>
       <c r="Q126" s="3" t="n"/>
       <c r="R126" s="3" t="n"/>
       <c r="S126" s="3" t="n"/>
       <c r="T126" s="3" t="n"/>
       <c r="U126" s="3" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
         <is>
-          <t>6807</t>
+          <t>6809</t>
         </is>
       </c>
       <c r="B127" s="3" t="n"/>
@@ -5969,9 +5996,7 @@
       <c r="I127" s="3" t="n"/>
       <c r="J127" s="3" t="n"/>
       <c r="K127" s="3" t="n"/>
-      <c r="L127" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="L127" s="3" t="n"/>
       <c r="M127" s="3" t="n"/>
       <c r="N127" s="3" t="n"/>
       <c r="O127" s="3" t="n">
@@ -5983,13 +6008,13 @@
       <c r="S127" s="3" t="n"/>
       <c r="T127" s="3" t="n"/>
       <c r="U127" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="3" t="inlineStr">
         <is>
-          <t>6809</t>
+          <t>6810</t>
         </is>
       </c>
       <c r="B128" s="3" t="n"/>
@@ -6006,7 +6031,7 @@
       <c r="M128" s="3" t="n"/>
       <c r="N128" s="3" t="n"/>
       <c r="O128" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="P128" s="3" t="n"/>
       <c r="Q128" s="3" t="n"/>
@@ -6014,13 +6039,13 @@
       <c r="S128" s="3" t="n"/>
       <c r="T128" s="3" t="n"/>
       <c r="U128" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="3" t="inlineStr">
         <is>
-          <t>6810</t>
+          <t>6815</t>
         </is>
       </c>
       <c r="B129" s="3" t="n"/>
@@ -6036,22 +6061,22 @@
       <c r="L129" s="3" t="n"/>
       <c r="M129" s="3" t="n"/>
       <c r="N129" s="3" t="n"/>
-      <c r="O129" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="O129" s="3" t="n"/>
       <c r="P129" s="3" t="n"/>
-      <c r="Q129" s="3" t="n"/>
+      <c r="Q129" s="3" t="n">
+        <v>6</v>
+      </c>
       <c r="R129" s="3" t="n"/>
       <c r="S129" s="3" t="n"/>
       <c r="T129" s="3" t="n"/>
       <c r="U129" s="3" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="3" t="inlineStr">
         <is>
-          <t>6815</t>
+          <t>6832</t>
         </is>
       </c>
       <c r="B130" s="3" t="n"/>
@@ -6070,19 +6095,19 @@
       <c r="O130" s="3" t="n"/>
       <c r="P130" s="3" t="n"/>
       <c r="Q130" s="3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="R130" s="3" t="n"/>
       <c r="S130" s="3" t="n"/>
       <c r="T130" s="3" t="n"/>
       <c r="U130" s="3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="3" t="inlineStr">
         <is>
-          <t>6832</t>
+          <t>6835</t>
         </is>
       </c>
       <c r="B131" s="3" t="n"/>
@@ -6113,7 +6138,7 @@
     <row r="132">
       <c r="A132" s="3" t="inlineStr">
         <is>
-          <t>6835</t>
+          <t>6900</t>
         </is>
       </c>
       <c r="B132" s="3" t="n"/>
@@ -6123,28 +6148,30 @@
       <c r="F132" s="3" t="n"/>
       <c r="G132" s="3" t="n"/>
       <c r="H132" s="3" t="n"/>
-      <c r="I132" s="3" t="n"/>
+      <c r="I132" s="3" t="n">
+        <v>21</v>
+      </c>
       <c r="J132" s="3" t="n"/>
       <c r="K132" s="3" t="n"/>
       <c r="L132" s="3" t="n"/>
       <c r="M132" s="3" t="n"/>
       <c r="N132" s="3" t="n"/>
       <c r="O132" s="3" t="n"/>
-      <c r="P132" s="3" t="n"/>
-      <c r="Q132" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="P132" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q132" s="3" t="n"/>
       <c r="R132" s="3" t="n"/>
       <c r="S132" s="3" t="n"/>
       <c r="T132" s="3" t="n"/>
       <c r="U132" s="3" t="n">
-        <v>4</v>
+        <v>22</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="3" t="inlineStr">
         <is>
-          <t>6900</t>
+          <t>6901</t>
         </is>
       </c>
       <c r="B133" s="3" t="n"/>
@@ -6154,15 +6181,17 @@
       <c r="F133" s="3" t="n"/>
       <c r="G133" s="3" t="n"/>
       <c r="H133" s="3" t="n"/>
-      <c r="I133" s="3" t="n">
-        <v>21</v>
-      </c>
+      <c r="I133" s="3" t="n"/>
       <c r="J133" s="3" t="n"/>
       <c r="K133" s="3" t="n"/>
-      <c r="L133" s="3" t="n"/>
+      <c r="L133" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="M133" s="3" t="n"/>
       <c r="N133" s="3" t="n"/>
-      <c r="O133" s="3" t="n"/>
+      <c r="O133" s="3" t="n">
+        <v>13</v>
+      </c>
       <c r="P133" s="3" t="n">
         <v>1</v>
       </c>
@@ -6171,13 +6200,13 @@
       <c r="S133" s="3" t="n"/>
       <c r="T133" s="3" t="n"/>
       <c r="U133" s="3" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="3" t="inlineStr">
         <is>
-          <t>6901</t>
+          <t>6902</t>
         </is>
       </c>
       <c r="B134" s="3" t="n"/>
@@ -6191,12 +6220,12 @@
       <c r="J134" s="3" t="n"/>
       <c r="K134" s="3" t="n"/>
       <c r="L134" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M134" s="3" t="n"/>
       <c r="N134" s="3" t="n"/>
       <c r="O134" s="3" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="P134" s="3" t="n">
         <v>1</v>
@@ -6206,41 +6235,6 @@
       <c r="S134" s="3" t="n"/>
       <c r="T134" s="3" t="n"/>
       <c r="U134" s="3" t="n">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" s="3" t="inlineStr">
-        <is>
-          <t>6902</t>
-        </is>
-      </c>
-      <c r="B135" s="3" t="n"/>
-      <c r="C135" s="3" t="n"/>
-      <c r="D135" s="3" t="n"/>
-      <c r="E135" s="3" t="n"/>
-      <c r="F135" s="3" t="n"/>
-      <c r="G135" s="3" t="n"/>
-      <c r="H135" s="3" t="n"/>
-      <c r="I135" s="3" t="n"/>
-      <c r="J135" s="3" t="n"/>
-      <c r="K135" s="3" t="n"/>
-      <c r="L135" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="M135" s="3" t="n"/>
-      <c r="N135" s="3" t="n"/>
-      <c r="O135" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="P135" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q135" s="3" t="n"/>
-      <c r="R135" s="3" t="n"/>
-      <c r="S135" s="3" t="n"/>
-      <c r="T135" s="3" t="n"/>
-      <c r="U135" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -6327,17 +6321,17 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Missing - OMi part not in Air-Way</t>
+          <t>Needs one specific item (see note)</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>OMi 0304-C-xx is a JIC CAP nut (OMi: "04 JIC Cap Nut"), not the Air-Way 0304 standard nut - needs a cap source (Brennan 0304-C STEPs or AN929) + the female JIC port per size</t>
+          <t xml:space="preserve">OMi-filled 2026-10-02 (was BUILD-MISSING: no Air-Way row): Brennan TFA catalog p65 prints </t>
         </is>
       </c>
     </row>
@@ -6364,17 +6358,17 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Missing - OMi part not in Air-Way</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>OMi 0304-C-xx is a JIC CAP nut (OMi: "04 JIC Cap Nut"), not the Air-Way 0304 standard nut - needs a cap source (Brennan 0304-C STEPs or AN929) + the female JIC port per size</t>
+          <t>master 0304</t>
         </is>
       </c>
     </row>
@@ -6401,17 +6395,17 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Missing - OMi part not in Air-Way</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>OMi 0304-C-xx is a JIC CAP nut (OMi: "04 JIC Cap Nut"), not the Air-Way 0304 standard nut - needs a cap source (Brennan 0304-C STEPs or AN929) + the female JIC port per size</t>
+          <t>master 0304</t>
         </is>
       </c>
     </row>
@@ -6438,17 +6432,17 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Missing - OMi part not in Air-Way</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>OMi 0304-C-xx is a JIC CAP nut (OMi: "04 JIC Cap Nut"), not the Air-Way 0304 standard nut - needs a cap source (Brennan 0304-C STEPs or AN929) + the female JIC port per size</t>
+          <t>master 0304</t>
         </is>
       </c>
     </row>
@@ -6475,17 +6469,17 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Missing - OMi part not in Air-Way</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>OMi 0304-C-xx is a JIC CAP nut (OMi: "04 JIC Cap Nut"), not the Air-Way 0304 standard nut - needs a cap source (Brennan 0304-C STEPs or AN929) + the female JIC port per size</t>
+          <t>master 0304</t>
         </is>
       </c>
     </row>
@@ -6512,17 +6506,17 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Missing - OMi part not in Air-Way</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>OMi 0304-C-xx is a JIC CAP nut (OMi: "04 JIC Cap Nut"), not the Air-Way 0304 standard nut - needs a cap source (Brennan 0304-C STEPs or AN929) + the female JIC port per size</t>
+          <t>master 0304</t>
         </is>
       </c>
     </row>
@@ -6549,17 +6543,17 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Missing - OMi part not in Air-Way</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>OMi 0304-C-xx is a JIC CAP nut (OMi: "04 JIC Cap Nut"), not the Air-Way 0304 standard nut - needs a cap source (Brennan 0304-C STEPs or AN929) + the female JIC port per size</t>
+          <t>master 0304</t>
         </is>
       </c>
     </row>
@@ -6586,17 +6580,17 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Missing - OMi part not in Air-Way</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>OMi 0304-C-xx is a JIC CAP nut (OMi: "04 JIC Cap Nut"), not the Air-Way 0304 standard nut - needs a cap source (Brennan 0304-C STEPs or AN929) + the female JIC port per size</t>
+          <t>master 0304</t>
         </is>
       </c>
     </row>
@@ -6623,17 +6617,17 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Missing - OMi part not in Air-Way</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>OMi 0304-C-xx is a JIC CAP nut (OMi: "04 JIC Cap Nut"), not the Air-Way 0304 standard nut - needs a cap source (Brennan 0304-C STEPs or AN929) + the female JIC port per size</t>
+          <t>master 0304</t>
         </is>
       </c>
     </row>
@@ -6660,17 +6654,17 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Missing - OMi part not in Air-Way</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>OMi 0304-C-xx is a JIC CAP nut (OMi: "04 JIC Cap Nut"), not the Air-Way 0304 standard nut - needs a cap source (Brennan 0304-C STEPs or AN929) + the female JIC port per size</t>
+          <t>master 0304</t>
         </is>
       </c>
     </row>
@@ -6697,17 +6691,17 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Missing - OMi part not in Air-Way</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>OMi 0304-C-xx is a JIC CAP nut (OMi: "04 JIC Cap Nut"), not the Air-Way 0304 standard nut - needs a cap source (Brennan 0304-C STEPs or AN929) + the female JIC port per size</t>
+          <t>master 0304</t>
         </is>
       </c>
     </row>
@@ -6734,17 +6728,17 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Missing - OMi part not in Air-Way</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>OMi 0304-C-xx is a JIC CAP nut (OMi: "04 JIC Cap Nut"), not the Air-Way 0304 standard nut - needs a cap source (Brennan 0304-C STEPs or AN929) + the female JIC port per size</t>
+          <t>master 0304</t>
         </is>
       </c>
     </row>
@@ -6771,17 +6765,17 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Missing - OMi part not in Air-Way</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>OMi 0304-C-xx is a JIC CAP nut (OMi: "04 JIC Cap Nut"), not the Air-Way 0304 standard nut - needs a cap source (Brennan 0304-C STEPs or AN929) + the female JIC port per size</t>
+          <t>master 0304</t>
         </is>
       </c>
     </row>
@@ -6808,15 +6802,19 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Missing - OMi part not in Air-Way</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr"/>
+          <t>Needs one specific item (see note)</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OMi-filled 2026-10-02 (was BUILD-MISSING: no Air-Way row): Brennan TFA catalog p65 prints </t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -6841,15 +6839,19 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Missing - OMi part not in Air-Way</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>master 0306</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -6874,15 +6876,19 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Missing - OMi part not in Air-Way</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>master 0306</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -6907,15 +6913,19 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Missing - OMi part not in Air-Way</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>master 0306</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -6940,15 +6950,19 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Missing - OMi part not in Air-Way</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>master 0306</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -6973,15 +6987,19 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>Missing - OMi part not in Air-Way</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>master 0306</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -7006,15 +7024,19 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Missing - OMi part not in Air-Way</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>master 0306</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -7039,15 +7061,19 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>Missing - OMi part not in Air-Way</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>master 0306</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -7072,15 +7098,19 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Missing - OMi part not in Air-Way</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>master 0306</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -7105,15 +7135,19 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>Missing - OMi part not in Air-Way</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>master 0306</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -7138,15 +7172,19 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>Missing - OMi part not in Air-Way</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>master 0306</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -7171,15 +7209,19 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>Missing - OMi part not in Air-Way</t>
-        </is>
-      </c>
-      <c r="G26" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>master 0306</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -10761,17 +10803,17 @@
       </c>
       <c r="E124" s="3" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F124" s="3" t="inlineStr">
         <is>
-          <t>Needs a Brennan STEP - female NPSM swivel size</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G124" s="3" t="inlineStr">
         <is>
-          <t>NPSM swivel -02: Brennan 1404-02-02 + NPSM elbow leg (my work)</t>
+          <t>master 1502</t>
         </is>
       </c>
     </row>
@@ -19069,12 +19111,12 @@
       </c>
       <c r="E372" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F372" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G372" s="3" t="inlineStr">
@@ -19101,22 +19143,22 @@
       </c>
       <c r="D373" s="3" t="inlineStr">
         <is>
-          <t>2404_FINAL</t>
+          <t>2404</t>
         </is>
       </c>
       <c r="E373" s="3" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F373" s="3" t="inlineStr">
         <is>
-          <t>Needs one specific item (see note)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G373" s="3" t="inlineStr">
         <is>
-          <t>BLOCKED: CB depth unsourced</t>
+          <t>master 2404</t>
         </is>
       </c>
     </row>
@@ -19143,12 +19185,12 @@
       </c>
       <c r="E374" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F374" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G374" s="3" t="inlineStr">
@@ -19180,12 +19222,12 @@
       </c>
       <c r="E375" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F375" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G375" s="3" t="inlineStr">
@@ -19217,12 +19259,12 @@
       </c>
       <c r="E376" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F376" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G376" s="3" t="inlineStr">
@@ -19254,12 +19296,12 @@
       </c>
       <c r="E377" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F377" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G377" s="3" t="inlineStr">
@@ -19291,12 +19333,12 @@
       </c>
       <c r="E378" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F378" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G378" s="3" t="inlineStr">
@@ -19328,12 +19370,12 @@
       </c>
       <c r="E379" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F379" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G379" s="3" t="inlineStr">
@@ -19365,12 +19407,12 @@
       </c>
       <c r="E380" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F380" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G380" s="3" t="inlineStr">
@@ -19402,12 +19444,12 @@
       </c>
       <c r="E381" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F381" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G381" s="3" t="inlineStr">
@@ -19439,12 +19481,12 @@
       </c>
       <c r="E382" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F382" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G382" s="3" t="inlineStr">
@@ -19476,12 +19518,12 @@
       </c>
       <c r="E383" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F383" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G383" s="3" t="inlineStr">
@@ -19513,12 +19555,12 @@
       </c>
       <c r="E384" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F384" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G384" s="3" t="inlineStr">
@@ -19550,12 +19592,12 @@
       </c>
       <c r="E385" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F385" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G385" s="3" t="inlineStr">
@@ -19587,12 +19629,12 @@
       </c>
       <c r="E386" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F386" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G386" s="3" t="inlineStr">
@@ -19624,12 +19666,12 @@
       </c>
       <c r="E387" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F387" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G387" s="3" t="inlineStr">
@@ -19661,12 +19703,12 @@
       </c>
       <c r="E388" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F388" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G388" s="3" t="inlineStr">
@@ -19693,22 +19735,22 @@
       </c>
       <c r="D389" s="3" t="inlineStr">
         <is>
-          <t>2404_FINAL</t>
+          <t>2404</t>
         </is>
       </c>
       <c r="E389" s="3" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F389" s="3" t="inlineStr">
         <is>
-          <t>Needs one specific item (see note)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G389" s="3" t="inlineStr">
         <is>
-          <t>BLOCKED: CB depth unsourced</t>
+          <t>master 2404</t>
         </is>
       </c>
     </row>
@@ -19735,12 +19777,12 @@
       </c>
       <c r="E390" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F390" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G390" s="3" t="inlineStr">
@@ -19772,12 +19814,12 @@
       </c>
       <c r="E391" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F391" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G391" s="3" t="inlineStr">
@@ -19809,12 +19851,12 @@
       </c>
       <c r="E392" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F392" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G392" s="3" t="inlineStr">
@@ -19846,12 +19888,12 @@
       </c>
       <c r="E393" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F393" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G393" s="3" t="inlineStr">
@@ -19883,12 +19925,12 @@
       </c>
       <c r="E394" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F394" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G394" s="3" t="inlineStr">
@@ -19920,12 +19962,12 @@
       </c>
       <c r="E395" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F395" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G395" s="3" t="inlineStr">
@@ -19957,12 +19999,12 @@
       </c>
       <c r="E396" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F396" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G396" s="3" t="inlineStr">
@@ -19994,12 +20036,12 @@
       </c>
       <c r="E397" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F397" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G397" s="3" t="inlineStr">
@@ -20031,12 +20073,12 @@
       </c>
       <c r="E398" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F398" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G398" s="3" t="inlineStr">
@@ -20068,12 +20110,12 @@
       </c>
       <c r="E399" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F399" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G399" s="3" t="inlineStr">
@@ -20105,12 +20147,12 @@
       </c>
       <c r="E400" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F400" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G400" s="3" t="inlineStr">
@@ -20142,12 +20184,12 @@
       </c>
       <c r="E401" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F401" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G401" s="3" t="inlineStr">
@@ -20179,12 +20221,12 @@
       </c>
       <c r="E402" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F402" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G402" s="3" t="inlineStr">
@@ -20216,12 +20258,12 @@
       </c>
       <c r="E403" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F403" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G403" s="3" t="inlineStr">
@@ -20253,12 +20295,12 @@
       </c>
       <c r="E404" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F404" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G404" s="3" t="inlineStr">
@@ -20290,12 +20332,12 @@
       </c>
       <c r="E405" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F405" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G405" s="3" t="inlineStr">
@@ -20327,12 +20369,12 @@
       </c>
       <c r="E406" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F406" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G406" s="3" t="inlineStr">
@@ -20364,12 +20406,12 @@
       </c>
       <c r="E407" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F407" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G407" s="3" t="inlineStr">
@@ -20401,12 +20443,12 @@
       </c>
       <c r="E408" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F408" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G408" s="3" t="inlineStr">
@@ -20438,12 +20480,12 @@
       </c>
       <c r="E409" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F409" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G409" s="3" t="inlineStr">
@@ -20470,22 +20512,22 @@
       </c>
       <c r="D410" s="3" t="inlineStr">
         <is>
-          <t>2404_FINAL</t>
+          <t>2404</t>
         </is>
       </c>
       <c r="E410" s="3" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F410" s="3" t="inlineStr">
         <is>
-          <t>Needs one specific item (see note)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G410" s="3" t="inlineStr">
         <is>
-          <t>BLOCKED: CB depth unsourced</t>
+          <t>master 2404</t>
         </is>
       </c>
     </row>
@@ -20512,12 +20554,12 @@
       </c>
       <c r="E411" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F411" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G411" s="3" t="inlineStr">
@@ -20549,12 +20591,12 @@
       </c>
       <c r="E412" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F412" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G412" s="3" t="inlineStr">
@@ -20586,12 +20628,12 @@
       </c>
       <c r="E413" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F413" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G413" s="3" t="inlineStr">
@@ -20623,12 +20665,12 @@
       </c>
       <c r="E414" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F414" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G414" s="3" t="inlineStr">
@@ -20660,12 +20702,12 @@
       </c>
       <c r="E415" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F415" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G415" s="3" t="inlineStr">
@@ -20697,12 +20739,12 @@
       </c>
       <c r="E416" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F416" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G416" s="3" t="inlineStr">
@@ -20734,12 +20776,12 @@
       </c>
       <c r="E417" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F417" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G417" s="3" t="inlineStr">
@@ -20771,12 +20813,12 @@
       </c>
       <c r="E418" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F418" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G418" s="3" t="inlineStr">
@@ -20808,12 +20850,12 @@
       </c>
       <c r="E419" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F419" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G419" s="3" t="inlineStr">
@@ -20840,22 +20882,22 @@
       </c>
       <c r="D420" s="3" t="inlineStr">
         <is>
-          <t>2404_FINAL</t>
+          <t>2404</t>
         </is>
       </c>
       <c r="E420" s="3" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F420" s="3" t="inlineStr">
         <is>
-          <t>Needs one specific item (see note)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G420" s="3" t="inlineStr">
         <is>
-          <t>BLOCKED: CB depth unsourced</t>
+          <t>master 2404</t>
         </is>
       </c>
     </row>
@@ -20882,12 +20924,12 @@
       </c>
       <c r="E421" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F421" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G421" s="3" t="inlineStr">
@@ -20919,12 +20961,12 @@
       </c>
       <c r="E422" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F422" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G422" s="3" t="inlineStr">
@@ -20993,12 +21035,12 @@
       </c>
       <c r="E424" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F424" s="3" t="inlineStr">
         <is>
-          <t>Built earlier - 2404 / 6400 masters (files not in 11_MASTERS)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G424" s="3" t="inlineStr">
@@ -21062,22 +21104,22 @@
       </c>
       <c r="D426" s="3" t="inlineStr">
         <is>
-          <t>2404L</t>
+          <t>2404</t>
         </is>
       </c>
       <c r="E426" s="3" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F426" s="3" t="inlineStr">
         <is>
-          <t>Needs one specific item (see note)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G426" s="3" t="inlineStr">
         <is>
-          <t>fold into the base master (your yes, 2026-09-25) - needs one Brennan STEP to see where the extra length goes: 2404-L-08-08</t>
+          <t>master 2404</t>
         </is>
       </c>
     </row>
@@ -21099,22 +21141,22 @@
       </c>
       <c r="D427" s="3" t="inlineStr">
         <is>
-          <t>2404L</t>
+          <t>2404</t>
         </is>
       </c>
       <c r="E427" s="3" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F427" s="3" t="inlineStr">
         <is>
-          <t>Needs one specific item (see note)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G427" s="3" t="inlineStr">
         <is>
-          <t>fold into the base master (your yes, 2026-09-25) - needs one Brennan STEP to see where the extra length goes: 2404-L-08-08</t>
+          <t>master 2404</t>
         </is>
       </c>
     </row>
@@ -21136,22 +21178,22 @@
       </c>
       <c r="D428" s="3" t="inlineStr">
         <is>
-          <t>2404L</t>
+          <t>2404</t>
         </is>
       </c>
       <c r="E428" s="3" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F428" s="3" t="inlineStr">
         <is>
-          <t>Needs one specific item (see note)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G428" s="3" t="inlineStr">
         <is>
-          <t>fold into the base master (your yes, 2026-09-25) - needs one Brennan STEP to see where the extra length goes: 2404-L-08-08</t>
+          <t>master 2404</t>
         </is>
       </c>
     </row>
@@ -21173,22 +21215,22 @@
       </c>
       <c r="D429" s="3" t="inlineStr">
         <is>
-          <t>2404L</t>
+          <t>2404</t>
         </is>
       </c>
       <c r="E429" s="3" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F429" s="3" t="inlineStr">
         <is>
-          <t>Needs one specific item (see note)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G429" s="3" t="inlineStr">
         <is>
-          <t>fold into the base master (your yes, 2026-09-25) - needs one Brennan STEP to see where the extra length goes: 2404-L-08-08</t>
+          <t>master 2404</t>
         </is>
       </c>
     </row>
@@ -21210,22 +21252,22 @@
       </c>
       <c r="D430" s="3" t="inlineStr">
         <is>
-          <t>2404L</t>
+          <t>2404</t>
         </is>
       </c>
       <c r="E430" s="3" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F430" s="3" t="inlineStr">
         <is>
-          <t>Needs one specific item (see note)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G430" s="3" t="inlineStr">
         <is>
-          <t>fold into the base master (your yes, 2026-09-25) - needs one Brennan STEP to see where the extra length goes: 2404-L-08-08</t>
+          <t>master 2404</t>
         </is>
       </c>
     </row>
@@ -28894,15 +28936,19 @@
       </c>
       <c r="E641" s="3" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F641" s="3" t="inlineStr">
         <is>
-          <t>Missing - Air-Way lists only the non-forged part (OMi sells -FG)</t>
-        </is>
-      </c>
-      <c r="G641" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G641" s="3" t="inlineStr">
+        <is>
+          <t>master 2504</t>
+        </is>
+      </c>
     </row>
     <row r="642">
       <c r="A642" s="3" t="inlineStr">
@@ -28927,15 +28973,19 @@
       </c>
       <c r="E642" s="3" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F642" s="3" t="inlineStr">
         <is>
-          <t>Missing - Air-Way lists only the non-forged part (OMi sells -FG)</t>
-        </is>
-      </c>
-      <c r="G642" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G642" s="3" t="inlineStr">
+        <is>
+          <t>master 2504</t>
+        </is>
+      </c>
     </row>
     <row r="643">
       <c r="A643" s="3" t="inlineStr">
@@ -28960,15 +29010,19 @@
       </c>
       <c r="E643" s="3" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F643" s="3" t="inlineStr">
         <is>
-          <t>Missing - Air-Way lists only the non-forged part (OMi sells -FG)</t>
-        </is>
-      </c>
-      <c r="G643" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G643" s="3" t="inlineStr">
+        <is>
+          <t>master 2504</t>
+        </is>
+      </c>
     </row>
     <row r="644">
       <c r="A644" s="3" t="inlineStr">
@@ -28993,15 +29047,19 @@
       </c>
       <c r="E644" s="3" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F644" s="3" t="inlineStr">
         <is>
-          <t>Missing - Air-Way lists only the non-forged part (OMi sells -FG)</t>
-        </is>
-      </c>
-      <c r="G644" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G644" s="3" t="inlineStr">
+        <is>
+          <t>master 2504</t>
+        </is>
+      </c>
     </row>
     <row r="645">
       <c r="A645" s="3" t="inlineStr">
@@ -29026,15 +29084,19 @@
       </c>
       <c r="E645" s="3" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="F645" s="3" t="inlineStr">
         <is>
-          <t>Missing - Air-Way lists only the non-forged part (OMi sells -FG)</t>
-        </is>
-      </c>
-      <c r="G645" s="3" t="inlineStr"/>
+          <t>Needs one specific item (see note)</t>
+        </is>
+      </c>
+      <c r="G645" s="3" t="inlineStr">
+        <is>
+          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series (e.g. 1501 N</t>
+        </is>
+      </c>
     </row>
     <row r="646">
       <c r="A646" s="3" t="inlineStr">
@@ -29059,15 +29121,19 @@
       </c>
       <c r="E646" s="3" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F646" s="3" t="inlineStr">
         <is>
-          <t>Missing - Air-Way lists only the non-forged part (OMi sells -FG)</t>
-        </is>
-      </c>
-      <c r="G646" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G646" s="3" t="inlineStr">
+        <is>
+          <t>master 2505</t>
+        </is>
+      </c>
     </row>
     <row r="647">
       <c r="A647" s="3" t="inlineStr">
@@ -29092,15 +29158,19 @@
       </c>
       <c r="E647" s="3" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="F647" s="3" t="inlineStr">
         <is>
-          <t>Missing - Air-Way lists only the non-forged part (OMi sells -FG)</t>
-        </is>
-      </c>
-      <c r="G647" s="3" t="inlineStr"/>
+          <t>Needs one specific item (see note)</t>
+        </is>
+      </c>
+      <c r="G647" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-02 (JIC-TEES): stays MISSING ONLY for the female port (TAPDRILL@BORE, PORTDEPTH@BO</t>
+        </is>
+      </c>
     </row>
     <row r="648">
       <c r="A648" s="3" t="inlineStr">
@@ -30412,15 +30482,19 @@
       </c>
       <c r="E683" s="3" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F683" s="3" t="inlineStr">
         <is>
-          <t>Missing - Air-Way lists only the non-forged part (OMi sells -FG)</t>
-        </is>
-      </c>
-      <c r="G683" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G683" s="3" t="inlineStr">
+        <is>
+          <t>master 2606</t>
+        </is>
+      </c>
     </row>
     <row r="684">
       <c r="A684" s="3" t="inlineStr">
@@ -30445,15 +30519,19 @@
       </c>
       <c r="E684" s="3" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F684" s="3" t="inlineStr">
         <is>
-          <t>Missing - Air-Way lists only the non-forged part (OMi sells -FG)</t>
-        </is>
-      </c>
-      <c r="G684" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G684" s="3" t="inlineStr">
+        <is>
+          <t>master 2606</t>
+        </is>
+      </c>
     </row>
     <row r="685">
       <c r="A685" s="3" t="inlineStr">
@@ -30478,15 +30556,19 @@
       </c>
       <c r="E685" s="3" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F685" s="3" t="inlineStr">
         <is>
-          <t>Missing - Air-Way lists only the non-forged part (OMi sells -FG)</t>
-        </is>
-      </c>
-      <c r="G685" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G685" s="3" t="inlineStr">
+        <is>
+          <t>master 2606</t>
+        </is>
+      </c>
     </row>
     <row r="686">
       <c r="A686" s="3" t="inlineStr">
@@ -30511,15 +30593,19 @@
       </c>
       <c r="E686" s="3" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F686" s="3" t="inlineStr">
         <is>
-          <t>Missing - OMi part not in Air-Way</t>
-        </is>
-      </c>
-      <c r="G686" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G686" s="3" t="inlineStr">
+        <is>
+          <t>master 2606</t>
+        </is>
+      </c>
     </row>
     <row r="687">
       <c r="A687" s="3" t="inlineStr">
@@ -30544,15 +30630,19 @@
       </c>
       <c r="E687" s="3" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F687" s="3" t="inlineStr">
         <is>
-          <t>Missing - Air-Way lists only the non-forged part (OMi sells -FG)</t>
-        </is>
-      </c>
-      <c r="G687" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G687" s="3" t="inlineStr">
+        <is>
+          <t>master 2606</t>
+        </is>
+      </c>
     </row>
     <row r="688">
       <c r="A688" s="3" t="inlineStr">
@@ -30577,15 +30667,19 @@
       </c>
       <c r="E688" s="3" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F688" s="3" t="inlineStr">
         <is>
-          <t>Missing - OMi part not in Air-Way</t>
-        </is>
-      </c>
-      <c r="G688" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G688" s="3" t="inlineStr">
+        <is>
+          <t>master 2609</t>
+        </is>
+      </c>
     </row>
     <row r="689">
       <c r="A689" s="3" t="inlineStr">
@@ -30610,15 +30704,19 @@
       </c>
       <c r="E689" s="3" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F689" s="3" t="inlineStr">
         <is>
-          <t>Missing - Air-Way lists only the non-forged part (OMi sells -FG)</t>
-        </is>
-      </c>
-      <c r="G689" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G689" s="3" t="inlineStr">
+        <is>
+          <t>master 2611</t>
+        </is>
+      </c>
     </row>
     <row r="690">
       <c r="A690" s="3" t="inlineStr">
@@ -30643,15 +30741,19 @@
       </c>
       <c r="E690" s="3" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F690" s="3" t="inlineStr">
         <is>
-          <t>Missing - OMi part not in Air-Way</t>
-        </is>
-      </c>
-      <c r="G690" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G690" s="3" t="inlineStr">
+        <is>
+          <t>master 2611</t>
+        </is>
+      </c>
     </row>
     <row r="691">
       <c r="A691" s="3" t="inlineStr">
@@ -30676,15 +30778,19 @@
       </c>
       <c r="E691" s="3" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>F5</t>
         </is>
       </c>
       <c r="F691" s="3" t="inlineStr">
         <is>
-          <t>Missing - Air-Way lists only the non-forged part (OMi sells -FG)</t>
-        </is>
-      </c>
-      <c r="G691" s="3" t="inlineStr"/>
+          <t>Missing - Air-Way cell blank / other</t>
+        </is>
+      </c>
+      <c r="G691" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-02 (JIC-TEES): stays MISSING - OMi gives no body dimensions for this part (M1@DRIVE, N5@DRIV</t>
+        </is>
+      </c>
     </row>
     <row r="692">
       <c r="A692" s="3" t="inlineStr">
@@ -58767,15 +58873,19 @@
       </c>
       <c r="E1478" s="3" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F1478" s="3" t="inlineStr">
         <is>
-          <t>Missing - Air-Way lists only the non-forged part (OMi sells -FG)</t>
-        </is>
-      </c>
-      <c r="G1478" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G1478" s="3" t="inlineStr">
+        <is>
+          <t>master 6500</t>
+        </is>
+      </c>
     </row>
     <row r="1479">
       <c r="A1479" s="3" t="inlineStr">
@@ -59133,15 +59243,19 @@
       </c>
       <c r="E1488" s="3" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F1488" s="3" t="inlineStr">
         <is>
-          <t>Missing - Air-Way lists only the non-forged part (OMi sells -FG)</t>
-        </is>
-      </c>
-      <c r="G1488" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G1488" s="3" t="inlineStr">
+        <is>
+          <t>master 6500</t>
+        </is>
+      </c>
     </row>
     <row r="1489">
       <c r="A1489" s="3" t="inlineStr">
@@ -59203,15 +59317,19 @@
       </c>
       <c r="E1490" s="3" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F1490" s="3" t="inlineStr">
         <is>
-          <t>Missing - Air-Way lists only the non-forged part (OMi sells -FG)</t>
-        </is>
-      </c>
-      <c r="G1490" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G1490" s="3" t="inlineStr">
+        <is>
+          <t>master 6500</t>
+        </is>
+      </c>
     </row>
     <row r="1491">
       <c r="A1491" s="3" t="inlineStr">
@@ -59236,15 +59354,19 @@
       </c>
       <c r="E1491" s="3" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F1491" s="3" t="inlineStr">
         <is>
-          <t>Missing - Air-Way lists only the non-forged part (OMi sells -FG)</t>
-        </is>
-      </c>
-      <c r="G1491" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G1491" s="3" t="inlineStr">
+        <is>
+          <t>master 6500</t>
+        </is>
+      </c>
     </row>
     <row r="1492">
       <c r="A1492" s="3" t="inlineStr">
@@ -59511,20 +59633,24 @@
       </c>
       <c r="D1499" s="3" t="inlineStr">
         <is>
-          <t>6500L</t>
+          <t>6500</t>
         </is>
       </c>
       <c r="E1499" s="3" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F1499" s="3" t="inlineStr">
         <is>
-          <t>Missing - Air-Way lists only the non-forged part (OMi sells -FG)</t>
-        </is>
-      </c>
-      <c r="G1499" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G1499" s="3" t="inlineStr">
+        <is>
+          <t>master 6500</t>
+        </is>
+      </c>
     </row>
     <row r="1500">
       <c r="A1500" s="3" t="inlineStr">
@@ -59544,20 +59670,24 @@
       </c>
       <c r="D1500" s="3" t="inlineStr">
         <is>
-          <t>6500L</t>
+          <t>6500</t>
         </is>
       </c>
       <c r="E1500" s="3" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F1500" s="3" t="inlineStr">
         <is>
-          <t>Missing - Air-Way lists only the non-forged part (OMi sells -FG)</t>
-        </is>
-      </c>
-      <c r="G1500" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G1500" s="3" t="inlineStr">
+        <is>
+          <t>master 6500</t>
+        </is>
+      </c>
     </row>
     <row r="1501">
       <c r="A1501" s="3" t="inlineStr">
@@ -59577,20 +59707,24 @@
       </c>
       <c r="D1501" s="3" t="inlineStr">
         <is>
-          <t>6500L</t>
+          <t>6500</t>
         </is>
       </c>
       <c r="E1501" s="3" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F1501" s="3" t="inlineStr">
         <is>
-          <t>Missing - Air-Way lists only the non-forged part (OMi sells -FG)</t>
-        </is>
-      </c>
-      <c r="G1501" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G1501" s="3" t="inlineStr">
+        <is>
+          <t>master 6500</t>
+        </is>
+      </c>
     </row>
     <row r="1502">
       <c r="A1502" s="3" t="inlineStr">
@@ -59610,20 +59744,24 @@
       </c>
       <c r="D1502" s="3" t="inlineStr">
         <is>
-          <t>6500L</t>
+          <t>6500</t>
         </is>
       </c>
       <c r="E1502" s="3" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F1502" s="3" t="inlineStr">
         <is>
-          <t>Missing - Air-Way lists only the non-forged part (OMi sells -FG)</t>
-        </is>
-      </c>
-      <c r="G1502" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G1502" s="3" t="inlineStr">
+        <is>
+          <t>master 6500</t>
+        </is>
+      </c>
     </row>
     <row r="1503">
       <c r="A1503" s="3" t="inlineStr">
@@ -59643,20 +59781,24 @@
       </c>
       <c r="D1503" s="3" t="inlineStr">
         <is>
-          <t>6500L</t>
+          <t>6500</t>
         </is>
       </c>
       <c r="E1503" s="3" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F1503" s="3" t="inlineStr">
         <is>
-          <t>Missing - Air-Way lists only the non-forged part (OMi sells -FG)</t>
-        </is>
-      </c>
-      <c r="G1503" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G1503" s="3" t="inlineStr">
+        <is>
+          <t>master 6500</t>
+        </is>
+      </c>
     </row>
     <row r="1504">
       <c r="A1504" s="3" t="inlineStr">
@@ -59792,15 +59934,19 @@
       </c>
       <c r="E1507" s="3" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F1507" s="3" t="inlineStr">
         <is>
-          <t>Missing - Air-Way lists only the non-forged part (OMi sells -FG)</t>
-        </is>
-      </c>
-      <c r="G1507" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G1507" s="3" t="inlineStr">
+        <is>
+          <t>master 6501</t>
+        </is>
+      </c>
     </row>
     <row r="1508">
       <c r="A1508" s="3" t="inlineStr">
@@ -59973,15 +60119,19 @@
       </c>
       <c r="E1512" s="3" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F1512" s="3" t="inlineStr">
         <is>
-          <t>Missing - OMi part not in Air-Way</t>
-        </is>
-      </c>
-      <c r="G1512" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G1512" s="3" t="inlineStr">
+        <is>
+          <t>master 6501</t>
+        </is>
+      </c>
     </row>
     <row r="1513">
       <c r="A1513" s="3" t="inlineStr">
@@ -60006,15 +60156,19 @@
       </c>
       <c r="E1513" s="3" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F1513" s="3" t="inlineStr">
         <is>
-          <t>Missing - Air-Way lists only the non-forged part (OMi sells -FG)</t>
-        </is>
-      </c>
-      <c r="G1513" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G1513" s="3" t="inlineStr">
+        <is>
+          <t>master 6501</t>
+        </is>
+      </c>
     </row>
     <row r="1514">
       <c r="A1514" s="3" t="inlineStr">
@@ -62068,15 +62222,19 @@
       </c>
       <c r="E1571" s="3" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F1571" s="3" t="inlineStr">
         <is>
-          <t>Missing - OMi part not in Air-Way</t>
-        </is>
-      </c>
-      <c r="G1571" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G1571" s="3" t="inlineStr">
+        <is>
+          <t>master 6505</t>
+        </is>
+      </c>
     </row>
     <row r="1572">
       <c r="A1572" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Batch 18 shipped: Air-Way first, ORFS masters, O-rings, A14, held roots fixed
- Air-Way first (26 roots, 320 cells + 4 Brennan cells; the 40 Triveni cells as Air-Way)
- 50 FS masters + O-ring master 4000; A14 1603-08-08-08-FG
- held roots 1700RC 1800 1703 4503 4603 fixed (QA #177); 5404N still held (QA #178)
- review PDFs + check (no AW/BI conflict); BLOCKED_NEEDS list
- live tools = tools_b18; post-ship verify 0 BAD; QA_Log #176-#178, coverage, status docs

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/00_DOCS/OMi_Coverage_2026-09-24.xlsx
+++ b/00_DOCS/OMi_Coverage_2026-09-24.xlsx
@@ -484,7 +484,7 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>1300</v>
+        <v>1339</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
@@ -684,7 +684,7 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
@@ -704,7 +704,7 @@
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
@@ -784,7 +784,7 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>134</v>
+        <v>113</v>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
@@ -955,7 +955,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1045,42 +1045,42 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>adjustable ORB stud (nut/washer) sizes + a new module</t>
+          <t>Needs one specific item (see note)</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>adjustable ORB stud + locknut (4603)</t>
+          <t>Air-Way 3051 prints one leg length N and the hex W</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>6801-XX-XX-NWO-FG per ORB size</t>
+          <t>3051</t>
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>4603-04-04-NWO-FG 4603-06-06-NWO-FG 4603-08-08-NWO-FG 4603-12-12-NWO-FG 4603-16-16-NWO-FG</t>
+          <t>3051-04-04 3051-06-06 3051-08-08 3051-12-12</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Needs one specific item (see note)</t>
+          <t>adjustable ORB stud (nut/washer) sizes + a new module</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Air-Way 3051 prints one leg length N and the hex W</t>
+          <t>adjustable ORB stud + locknut (6801L)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>3051</t>
+          <t>6801-XX-XX-NWO-FG per ORB size</t>
         </is>
       </c>
       <c r="D5" s="3" t="n">
@@ -1088,7 +1088,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>3051-04-04 3051-06-06 3051-08-08 3051-12-12</t>
+          <t>6801-L-04-04-NWO-FG 6801-L-06-06-NWO-FG 6801-L-08-08-NWO-FG 6801-L-12-12-NWO-FG</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>adjustable ORB stud + locknut (6801L)</t>
+          <t>adjustable ORB stud + locknut (6801LL)</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -1109,11 +1109,11 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>6801-L-04-04-NWO-FG 6801-L-06-06-NWO-FG 6801-L-08-08-NWO-FG 6801-L-12-12-NWO-FG</t>
+          <t>6801-LL-04-04-NWO-FG 6801-LL-06-06-NWO-FG 6801-LL-08-08-NWO-FG</t>
         </is>
       </c>
     </row>
@@ -1125,7 +1125,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>adjustable ORB stud + locknut (6801LL)</t>
+          <t>adjustable ORB stud + locknut (6805)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>6801-LL-04-04-NWO-FG 6801-LL-06-06-NWO-FG 6801-LL-08-08-NWO-FG</t>
+          <t>6805-06-04-NWO-FG 6805-08-06-NWO-FG 6805-12-12-NWO-FG</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>adjustable ORB stud + locknut (6805)</t>
+          <t>adjustable ORB stud + locknut (6901)</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -1163,57 +1163,57 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>6805-06-04-NWO-FG 6805-08-06-NWO-FG 6805-12-12-NWO-FG</t>
+          <t>6901-06-04-NWO-FG 6901-06-06-NWO-FG 6901-10-08-NWO-FG</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>adjustable ORB stud (nut/washer) sizes + a new module</t>
+          <t>Needs one specific item (see note)</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>adjustable ORB stud + locknut (6901)</t>
+          <t>OMi-filled 2026-10-02 (was BUILD-MISSING</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>6801-XX-XX-NWO-FG per ORB size</t>
+          <t>TFA</t>
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>6901-06-04-NWO-FG 6901-06-06-NWO-FG 6901-10-08-NWO-FG</t>
+          <t>0304-C-02 0306-02</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Needs one specific item (see note)</t>
+          <t>female NPSM swivel size</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>OMi-filled 2026-10-02 (was BUILD-MISSING</t>
+          <t>NPSM swivel -02</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>TFA</t>
+          <t>1404-02-02</t>
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>0304-C-02 0306-02</t>
+          <t>1501-04-02-FG</t>
         </is>
       </c>
     </row>
@@ -1225,12 +1225,12 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>NPSM swivel -02</t>
+          <t>NPSM swivel -24</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>1404-02-02</t>
+          <t>1404-24-24</t>
         </is>
       </c>
       <c r="D11" s="3" t="n">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>1501-04-02-FG</t>
+          <t>1501-24-24-FG</t>
         </is>
       </c>
     </row>
@@ -1250,12 +1250,12 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>NPSM swivel -24</t>
+          <t>NPSM swivel -04</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>1404-24-24</t>
+          <t>1404-04-04</t>
         </is>
       </c>
       <c r="D12" s="3" t="n">
@@ -1263,24 +1263,24 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>1501-24-24-FG</t>
+          <t>1502-04-04-FG</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>female NPSM swivel size</t>
+          <t>female JIC port size</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>NPSM swivel -04</t>
+          <t>female JIC -16</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>1404-04-04</t>
+          <t>2406-16-xx</t>
         </is>
       </c>
       <c r="D13" s="3" t="n">
@@ -1288,24 +1288,24 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>1502-04-04-FG</t>
+          <t>2406-16-04</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Needs one specific item (see note)</t>
+          <t>female ORB port size</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>female ORB -20 port</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>catalog,</t>
+          <t>6404/6410</t>
         </is>
       </c>
       <c r="D14" s="3" t="n">
@@ -1313,24 +1313,24 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>1800-08-08</t>
+          <t>6410-32-20-O</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>female JIC port size</t>
+          <t>female ORB port size</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>female JIC -16</t>
+          <t>female ORB -24 port</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>2406-16-xx</t>
+          <t>6404/6410</t>
         </is>
       </c>
       <c r="D15" s="3" t="n">
@@ -1338,24 +1338,24 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>2406-16-04</t>
+          <t>6410-32-24-O</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>female ORB port size</t>
+          <t>adjustable ORB stud (nut/washer) sizes + a new module</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>female ORB -20 port</t>
+          <t>adjustable ORB stud + locknut (6802)</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>6404/6410</t>
+          <t>6801-XX-XX-NWO-FG per ORB size</t>
         </is>
       </c>
       <c r="D16" s="3" t="n">
@@ -1363,80 +1363,30 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>6410-32-20-O</t>
+          <t>6802-04-06-NWO-FG</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>female ORB port size</t>
+          <t>adjustable ORB stud (nut/washer) sizes + a new module</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>female ORB -24 port</t>
+          <t>adjustable ORB stud + locknut (6806)</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>6404/6410</t>
+          <t>6801-XX-XX-NWO-FG per ORB size</t>
         </is>
       </c>
       <c r="D17" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>6410-32-24-O</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>adjustable ORB stud (nut/washer) sizes + a new module</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>adjustable ORB stud + locknut (6802)</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>6801-XX-XX-NWO-FG per ORB size</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>6802-04-06-NWO-FG</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>adjustable ORB stud (nut/washer) sizes + a new module</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>adjustable ORB stud + locknut (6806)</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>6801-XX-XX-NWO-FG per ORB size</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
         <is>
           <t>6806-04-04-NWO-FG</t>
         </is>
@@ -1500,11 +1450,11 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>1502-08-08-FG 1504-24-24-FG 1603-08-08-08-FG 1704-32-32-FG 2500-06-04-FG 2500-08-06-FG 2500-12-08-FG 2500-12-10-FG 2501-LL-08-08-FG 2502-06-08-FG 2502-08-04-FG 2502-12-08-FG 2502-16-20-FG 2502-24-24-FG 5503-24-24-FG 5503-32-32-FG 5504-24-24-FG 5504-32-32-FG 5505-02-02-FG 5505-06-06-FG 5505-08-08-FG 5505-12-12-FG 5505-16-16-FG 5601-06-06-06-FG 5602-02-02-02-FG 5602-06-06-06-FG 5602-12-12-12-FG 5602-16-16-16-FG 5602-20-20-20-FG 5602-24-24-24-FG 5602-32-32-32-FG 5603-08-08-08-FG 5604-02-02-02-FG 5604-12-12-12-FG 5604-16-16-16-FG 5604-20-20-20-FG 5605-02-02-02-FG 5605-12-12-12-FG 5605-16-16-16-FG 5605-20-20-20-FG 5605-32-32-32-FG 5652-08-08-08-08-FG 5652-24-24-24-24-FG 6503-04-04-FG 6503-06-06-FG 6503-12-12-FG 6503-16-16-FG 6603-06-06-06-FG 6603-16-16-16-FG 6606-06-06-06-FG 6606-12-12-12-FG 6801-08-04-NWO-FG 6801-08-16-NWO-FG 6801-12-20-NWO-FG 6801-16-24-NWO-FG 6801-24-16-NWO-FG 6801-L-16-16-NWO-FG 6801-L-20-20-NWO-FG 6801-LL-12-12-NWO-FG 6801-LL-16-16-NWO-FG 6801-LL-20-20-NWO-FG 6802-06-10-NWO-FG 6802-08-12-NWO-FG 6803-08-08-06-NWO-FG 6803-08-08-10-NWO-FG 6803-24-24-24-NWO-FG 6804-24-24-24-NWO-FG 6805-04-02-NWO-FG 6805-04-04-NWO-FG 6805-06-06-NWO-FG 6805-08-08-NWO-FG 6805-10-08-NWO-FG 6805-12-08-NWO-FG 6805-16-12-NWO-FG 6805-16-16-NWO-FG 6805-20-20-NWO-FG 6806-06-04-NWO-FG 6806-06-06-NWO-FG 6806-08-06-NWO-FG 6806-08-08-NWO-FG 6806-10-08-NWO-FG 6806-12-12-NWO-FG 6806-16-16-NWO-FG 6806-20-20-NWO-FG 6806-24-24-NWO-FG 6807-04-04-NWO-FG 6807-08-06-NWO-FG 6807-08-08-NWO-FG 6807-12-12-NWO-FG 6809-10-10-NWO-FG 6809-12-12-NWO-FG 6809-16-16-NWO-FG 6809-20-20-NWO-FG 6810-12-12-NWO-FG 6901-04-04-NWO-FG 6901-04-06-NWO-FG 6901-06-08-NWO-FG 6901-10-12-NWO-FG 6901-12-06-NWO-FG 6901-12-08-NWO-FG 6901-12-12-NWO-FG 6901-12-16-NWO-FG 6901-16-12-NWO-FG 6901-16-16-NWO-FG 6901-20-16-NWO-FG 6901-20-20-NWO-FG 6901-24-24-NWO-FG 6902-04-04-NWO-FG 6902-06-04-NWO-FG 6902-06-06-NWO-FG 6902-08-06-NWO-FG 6902-08-08-NWO-FG 6902-10-08-NWO-FG 6902-10-12-NWO-FG 6902-16-16-NWO-FG</t>
+          <t>1502-08-08-FG 1504-24-24-FG 1704-32-32-FG 2500-06-04-FG 2500-08-06-FG 2500-12-08-FG 2500-12-10-FG 2501-LL-08-08-FG 2502-06-08-FG 2502-08-04-FG 2502-12-08-FG 2502-16-20-FG 2502-24-24-FG 5503-24-24-FG 5503-32-32-FG 5504-24-24-FG 5504-32-32-FG 5505-02-02-FG 5505-06-06-FG 5505-08-08-FG 5505-12-12-FG 5505-16-16-FG 5601-06-06-06-FG 5602-02-02-02-FG 5602-06-06-06-FG 5602-12-12-12-FG 5602-16-16-16-FG 5602-20-20-20-FG 5602-24-24-24-FG 5602-32-32-32-FG 5603-08-08-08-FG 5604-02-02-02-FG 5604-12-12-12-FG 5604-16-16-16-FG 5604-20-20-20-FG 5605-02-02-02-FG 5605-12-12-12-FG 5605-16-16-16-FG 5605-20-20-20-FG 5605-32-32-32-FG 5652-08-08-08-08-FG 5652-24-24-24-24-FG 6503-04-04-FG 6503-06-06-FG 6503-12-12-FG 6503-16-16-FG 6603-06-06-06-FG 6603-16-16-16-FG 6606-06-06-06-FG 6606-12-12-12-FG 6801-08-04-NWO-FG 6801-08-16-NWO-FG 6801-12-20-NWO-FG 6801-16-24-NWO-FG 6801-24-16-NWO-FG 6801-L-16-16-NWO-FG 6801-L-20-20-NWO-FG 6801-LL-12-12-NWO-FG 6801-LL-16-16-NWO-FG 6801-LL-20-20-NWO-FG 6802-06-10-NWO-FG 6802-08-12-NWO-FG 6803-08-08-06-NWO-FG 6803-08-08-10-NWO-FG 6803-24-24-24-NWO-FG 6804-24-24-24-NWO-FG 6805-04-02-NWO-FG 6805-04-04-NWO-FG 6805-06-06-NWO-FG 6805-08-08-NWO-FG 6805-10-08-NWO-FG 6805-12-08-NWO-FG 6805-16-12-NWO-FG 6805-16-16-NWO-FG 6805-20-20-NWO-FG 6806-06-04-NWO-FG 6806-06-06-NWO-FG 6806-08-06-NWO-FG 6806-08-08-NWO-FG 6806-10-08-NWO-FG 6806-12-12-NWO-FG 6806-16-16-NWO-FG 6806-20-20-NWO-FG 6806-24-24-NWO-FG 6807-04-04-NWO-FG 6807-08-06-NWO-FG 6807-08-08-NWO-FG 6807-12-12-NWO-FG 6809-10-10-NWO-FG 6809-12-12-NWO-FG 6809-16-16-NWO-FG 6809-20-20-NWO-FG 6810-12-12-NWO-FG 6901-04-04-NWO-FG 6901-04-06-NWO-FG 6901-06-08-NWO-FG 6901-10-12-NWO-FG 6901-12-06-NWO-FG 6901-12-08-NWO-FG 6901-12-12-NWO-FG 6901-12-16-NWO-FG 6901-16-12-NWO-FG 6901-16-16-NWO-FG 6901-20-16-NWO-FG 6901-20-20-NWO-FG 6901-24-24-NWO-FG 6902-04-04-NWO-FG 6902-06-04-NWO-FG 6902-06-06-NWO-FG 6902-08-06-NWO-FG 6902-08-08-NWO-FG 6902-10-08-NWO-FG 6902-10-12-NWO-FG 6902-16-16-NWO-FG</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2090,7 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C17" s="3" t="n"/>
       <c r="D17" s="3" t="n"/>
@@ -2154,9 +2104,7 @@
       <c r="L17" s="3" t="n"/>
       <c r="M17" s="3" t="n"/>
       <c r="N17" s="3" t="n"/>
-      <c r="O17" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="O17" s="3" t="n"/>
       <c r="P17" s="3" t="n"/>
       <c r="Q17" s="3" t="n"/>
       <c r="R17" s="3" t="n"/>
@@ -2185,9 +2133,7 @@
       <c r="J18" s="3" t="n"/>
       <c r="K18" s="3" t="n"/>
       <c r="L18" s="3" t="n"/>
-      <c r="M18" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="M18" s="3" t="n"/>
       <c r="N18" s="3" t="n"/>
       <c r="O18" s="3" t="n"/>
       <c r="P18" s="3" t="n"/>
@@ -2196,16 +2142,18 @@
       <c r="S18" s="3" t="n"/>
       <c r="T18" s="3" t="n"/>
       <c r="U18" s="3" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>1703</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="n"/>
+          <t>1700RC</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="C19" s="3" t="n"/>
       <c r="D19" s="3" t="n"/>
       <c r="E19" s="3" t="n"/>
@@ -2216,26 +2164,22 @@
       <c r="J19" s="3" t="n"/>
       <c r="K19" s="3" t="n"/>
       <c r="L19" s="3" t="n"/>
-      <c r="M19" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="M19" s="3" t="n"/>
       <c r="N19" s="3" t="n"/>
       <c r="O19" s="3" t="n"/>
-      <c r="P19" s="3" t="n">
-        <v>18</v>
-      </c>
+      <c r="P19" s="3" t="n"/>
       <c r="Q19" s="3" t="n"/>
       <c r="R19" s="3" t="n"/>
       <c r="S19" s="3" t="n"/>
       <c r="T19" s="3" t="n"/>
       <c r="U19" s="3" t="n">
-        <v>19</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>1704</t>
+          <t>1703</t>
         </is>
       </c>
       <c r="B20" s="3" t="n">
@@ -2253,24 +2197,22 @@
       <c r="L20" s="3" t="n"/>
       <c r="M20" s="3" t="n"/>
       <c r="N20" s="3" t="n"/>
-      <c r="O20" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="O20" s="3" t="n"/>
       <c r="P20" s="3" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="Q20" s="3" t="n"/>
       <c r="R20" s="3" t="n"/>
       <c r="S20" s="3" t="n"/>
       <c r="T20" s="3" t="n"/>
       <c r="U20" s="3" t="n">
-        <v>25</v>
+        <v>19</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>1724</t>
+          <t>1704</t>
         </is>
       </c>
       <c r="B21" s="3" t="n">
@@ -2288,25 +2230,29 @@
       <c r="L21" s="3" t="n"/>
       <c r="M21" s="3" t="n"/>
       <c r="N21" s="3" t="n"/>
-      <c r="O21" s="3" t="n"/>
-      <c r="P21" s="3" t="n"/>
-      <c r="Q21" s="3" t="n">
-        <v>6</v>
-      </c>
+      <c r="O21" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P21" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="Q21" s="3" t="n"/>
       <c r="R21" s="3" t="n"/>
       <c r="S21" s="3" t="n"/>
       <c r="T21" s="3" t="n"/>
       <c r="U21" s="3" t="n">
-        <v>7</v>
+        <v>25</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>1800</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="n"/>
+          <t>1724</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="C22" s="3" t="n"/>
       <c r="D22" s="3" t="n"/>
       <c r="E22" s="3" t="n"/>
@@ -2317,29 +2263,29 @@
       <c r="J22" s="3" t="n"/>
       <c r="K22" s="3" t="n"/>
       <c r="L22" s="3" t="n"/>
-      <c r="M22" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="M22" s="3" t="n"/>
       <c r="N22" s="3" t="n"/>
       <c r="O22" s="3" t="n"/>
       <c r="P22" s="3" t="n"/>
       <c r="Q22" s="3" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="R22" s="3" t="n"/>
       <c r="S22" s="3" t="n"/>
       <c r="T22" s="3" t="n"/>
       <c r="U22" s="3" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>1803</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="n"/>
+          <t>1800</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="C23" s="3" t="n"/>
       <c r="D23" s="3" t="n"/>
       <c r="E23" s="3" t="n"/>
@@ -2355,24 +2301,22 @@
       <c r="O23" s="3" t="n"/>
       <c r="P23" s="3" t="n"/>
       <c r="Q23" s="3" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="R23" s="3" t="n"/>
       <c r="S23" s="3" t="n"/>
       <c r="T23" s="3" t="n"/>
       <c r="U23" s="3" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>1804</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="n">
-        <v>1</v>
-      </c>
+          <t>1803</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n"/>
       <c r="C24" s="3" t="n"/>
       <c r="D24" s="3" t="n"/>
       <c r="E24" s="3" t="n"/>
@@ -2388,19 +2332,19 @@
       <c r="O24" s="3" t="n"/>
       <c r="P24" s="3" t="n"/>
       <c r="Q24" s="3" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="R24" s="3" t="n"/>
       <c r="S24" s="3" t="n"/>
       <c r="T24" s="3" t="n"/>
       <c r="U24" s="3" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>1824</t>
+          <t>1804</t>
         </is>
       </c>
       <c r="B25" s="3" t="n">
@@ -2421,22 +2365,24 @@
       <c r="O25" s="3" t="n"/>
       <c r="P25" s="3" t="n"/>
       <c r="Q25" s="3" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="R25" s="3" t="n"/>
       <c r="S25" s="3" t="n"/>
       <c r="T25" s="3" t="n"/>
       <c r="U25" s="3" t="n">
-        <v>6</v>
+        <v>22</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>1901</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="n"/>
+          <t>1824</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="C26" s="3" t="n"/>
       <c r="D26" s="3" t="n"/>
       <c r="E26" s="3" t="n"/>
@@ -2451,20 +2397,20 @@
       <c r="N26" s="3" t="n"/>
       <c r="O26" s="3" t="n"/>
       <c r="P26" s="3" t="n"/>
-      <c r="Q26" s="3" t="n"/>
+      <c r="Q26" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="R26" s="3" t="n"/>
       <c r="S26" s="3" t="n"/>
-      <c r="T26" s="3" t="n">
-        <v>10</v>
-      </c>
+      <c r="T26" s="3" t="n"/>
       <c r="U26" s="3" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="B27" s="3" t="n"/>
@@ -2486,16 +2432,16 @@
       <c r="R27" s="3" t="n"/>
       <c r="S27" s="3" t="n"/>
       <c r="T27" s="3" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="U27" s="3" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>1927-61</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="B28" s="3" t="n"/>
@@ -2517,16 +2463,16 @@
       <c r="R28" s="3" t="n"/>
       <c r="S28" s="3" t="n"/>
       <c r="T28" s="3" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="U28" s="3" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>1927-62</t>
+          <t>1927-61</t>
         </is>
       </c>
       <c r="B29" s="3" t="n"/>
@@ -2557,12 +2503,10 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>2403</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="n">
-        <v>39</v>
-      </c>
+          <t>1927-62</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n"/>
       <c r="C30" s="3" t="n"/>
       <c r="D30" s="3" t="n"/>
       <c r="E30" s="3" t="n"/>
@@ -2576,25 +2520,25 @@
       <c r="M30" s="3" t="n"/>
       <c r="N30" s="3" t="n"/>
       <c r="O30" s="3" t="n"/>
-      <c r="P30" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="P30" s="3" t="n"/>
       <c r="Q30" s="3" t="n"/>
       <c r="R30" s="3" t="n"/>
       <c r="S30" s="3" t="n"/>
-      <c r="T30" s="3" t="n"/>
+      <c r="T30" s="3" t="n">
+        <v>6</v>
+      </c>
       <c r="U30" s="3" t="n">
-        <v>40</v>
+        <v>6</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>2404</t>
+          <t>2403</t>
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>57</v>
+        <v>39</v>
       </c>
       <c r="C31" s="3" t="n"/>
       <c r="D31" s="3" t="n"/>
@@ -2609,22 +2553,26 @@
       <c r="M31" s="3" t="n"/>
       <c r="N31" s="3" t="n"/>
       <c r="O31" s="3" t="n"/>
-      <c r="P31" s="3" t="n"/>
+      <c r="P31" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="Q31" s="3" t="n"/>
       <c r="R31" s="3" t="n"/>
       <c r="S31" s="3" t="n"/>
       <c r="T31" s="3" t="n"/>
       <c r="U31" s="3" t="n">
-        <v>57</v>
+        <v>40</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>2404L</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="n"/>
+          <t>2404</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>57</v>
+      </c>
       <c r="C32" s="3" t="n"/>
       <c r="D32" s="3" t="n"/>
       <c r="E32" s="3" t="n"/>
@@ -2638,21 +2586,19 @@
       <c r="M32" s="3" t="n"/>
       <c r="N32" s="3" t="n"/>
       <c r="O32" s="3" t="n"/>
-      <c r="P32" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="P32" s="3" t="n"/>
       <c r="Q32" s="3" t="n"/>
       <c r="R32" s="3" t="n"/>
       <c r="S32" s="3" t="n"/>
       <c r="T32" s="3" t="n"/>
       <c r="U32" s="3" t="n">
-        <v>1</v>
+        <v>57</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>2404_FINAL</t>
+          <t>2404L</t>
         </is>
       </c>
       <c r="B33" s="3" t="n"/>
@@ -2666,29 +2612,27 @@
       <c r="J33" s="3" t="n"/>
       <c r="K33" s="3" t="n"/>
       <c r="L33" s="3" t="n"/>
-      <c r="M33" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="M33" s="3" t="n"/>
       <c r="N33" s="3" t="n"/>
       <c r="O33" s="3" t="n"/>
-      <c r="P33" s="3" t="n"/>
+      <c r="P33" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="Q33" s="3" t="n"/>
       <c r="R33" s="3" t="n"/>
       <c r="S33" s="3" t="n"/>
       <c r="T33" s="3" t="n"/>
       <c r="U33" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>2405</t>
-        </is>
-      </c>
-      <c r="B34" s="3" t="n">
-        <v>30</v>
-      </c>
+          <t>2404_FINAL</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n"/>
       <c r="C34" s="3" t="n"/>
       <c r="D34" s="3" t="n"/>
       <c r="E34" s="3" t="n"/>
@@ -2699,7 +2643,9 @@
       <c r="J34" s="3" t="n"/>
       <c r="K34" s="3" t="n"/>
       <c r="L34" s="3" t="n"/>
-      <c r="M34" s="3" t="n"/>
+      <c r="M34" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="N34" s="3" t="n"/>
       <c r="O34" s="3" t="n"/>
       <c r="P34" s="3" t="n"/>
@@ -2708,17 +2654,17 @@
       <c r="S34" s="3" t="n"/>
       <c r="T34" s="3" t="n"/>
       <c r="U34" s="3" t="n">
-        <v>30</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>2406</t>
+          <t>2405</t>
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="C35" s="3" t="n"/>
       <c r="D35" s="3" t="n"/>
@@ -2726,34 +2672,30 @@
       <c r="F35" s="3" t="n"/>
       <c r="G35" s="3" t="n"/>
       <c r="H35" s="3" t="n"/>
-      <c r="I35" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="I35" s="3" t="n"/>
       <c r="J35" s="3" t="n"/>
       <c r="K35" s="3" t="n"/>
       <c r="L35" s="3" t="n"/>
       <c r="M35" s="3" t="n"/>
       <c r="N35" s="3" t="n"/>
       <c r="O35" s="3" t="n"/>
-      <c r="P35" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="P35" s="3" t="n"/>
       <c r="Q35" s="3" t="n"/>
       <c r="R35" s="3" t="n"/>
       <c r="S35" s="3" t="n"/>
       <c r="T35" s="3" t="n"/>
       <c r="U35" s="3" t="n">
-        <v>51</v>
+        <v>30</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>2408</t>
+          <t>2406</t>
         </is>
       </c>
       <c r="B36" s="3" t="n">
-        <v>12</v>
+        <v>49</v>
       </c>
       <c r="C36" s="3" t="n"/>
       <c r="D36" s="3" t="n"/>
@@ -2761,31 +2703,35 @@
       <c r="F36" s="3" t="n"/>
       <c r="G36" s="3" t="n"/>
       <c r="H36" s="3" t="n"/>
-      <c r="I36" s="3" t="n"/>
+      <c r="I36" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="J36" s="3" t="n"/>
       <c r="K36" s="3" t="n"/>
       <c r="L36" s="3" t="n"/>
       <c r="M36" s="3" t="n"/>
       <c r="N36" s="3" t="n"/>
       <c r="O36" s="3" t="n"/>
-      <c r="P36" s="3" t="n"/>
+      <c r="P36" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="Q36" s="3" t="n"/>
-      <c r="R36" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="R36" s="3" t="n"/>
       <c r="S36" s="3" t="n"/>
       <c r="T36" s="3" t="n"/>
       <c r="U36" s="3" t="n">
-        <v>13</v>
+        <v>51</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>2500</t>
-        </is>
-      </c>
-      <c r="B37" s="3" t="n"/>
+          <t>2408</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>12</v>
+      </c>
       <c r="C37" s="3" t="n"/>
       <c r="D37" s="3" t="n"/>
       <c r="E37" s="3" t="n"/>
@@ -2798,27 +2744,25 @@
       <c r="L37" s="3" t="n"/>
       <c r="M37" s="3" t="n"/>
       <c r="N37" s="3" t="n"/>
-      <c r="O37" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="O37" s="3" t="n"/>
       <c r="P37" s="3" t="n"/>
       <c r="Q37" s="3" t="n"/>
-      <c r="R37" s="3" t="n"/>
+      <c r="R37" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="S37" s="3" t="n"/>
       <c r="T37" s="3" t="n"/>
       <c r="U37" s="3" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>2500HX</t>
-        </is>
-      </c>
-      <c r="B38" s="3" t="n">
-        <v>11</v>
-      </c>
+          <t>2500</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n"/>
       <c r="C38" s="3" t="n"/>
       <c r="D38" s="3" t="n"/>
       <c r="E38" s="3" t="n"/>
@@ -2831,24 +2775,26 @@
       <c r="L38" s="3" t="n"/>
       <c r="M38" s="3" t="n"/>
       <c r="N38" s="3" t="n"/>
-      <c r="O38" s="3" t="n"/>
+      <c r="O38" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="P38" s="3" t="n"/>
       <c r="Q38" s="3" t="n"/>
       <c r="R38" s="3" t="n"/>
       <c r="S38" s="3" t="n"/>
       <c r="T38" s="3" t="n"/>
       <c r="U38" s="3" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>2501</t>
+          <t>2500HX</t>
         </is>
       </c>
       <c r="B39" s="3" t="n">
-        <v>54</v>
+        <v>11</v>
       </c>
       <c r="C39" s="3" t="n"/>
       <c r="D39" s="3" t="n"/>
@@ -2863,24 +2809,24 @@
       <c r="M39" s="3" t="n"/>
       <c r="N39" s="3" t="n"/>
       <c r="O39" s="3" t="n"/>
-      <c r="P39" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="P39" s="3" t="n"/>
       <c r="Q39" s="3" t="n"/>
       <c r="R39" s="3" t="n"/>
       <c r="S39" s="3" t="n"/>
       <c r="T39" s="3" t="n"/>
       <c r="U39" s="3" t="n">
-        <v>55</v>
+        <v>11</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>2501LL</t>
-        </is>
-      </c>
-      <c r="B40" s="3" t="n"/>
+          <t>2501</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>54</v>
+      </c>
       <c r="C40" s="3" t="n"/>
       <c r="D40" s="3" t="n"/>
       <c r="E40" s="3" t="n"/>
@@ -2893,22 +2839,22 @@
       <c r="L40" s="3" t="n"/>
       <c r="M40" s="3" t="n"/>
       <c r="N40" s="3" t="n"/>
-      <c r="O40" s="3" t="n">
+      <c r="O40" s="3" t="n"/>
+      <c r="P40" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="P40" s="3" t="n"/>
       <c r="Q40" s="3" t="n"/>
       <c r="R40" s="3" t="n"/>
       <c r="S40" s="3" t="n"/>
       <c r="T40" s="3" t="n"/>
       <c r="U40" s="3" t="n">
-        <v>1</v>
+        <v>55</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>2502</t>
+          <t>2501LL</t>
         </is>
       </c>
       <c r="B41" s="3" t="n"/>
@@ -2925,28 +2871,24 @@
       <c r="M41" s="3" t="n"/>
       <c r="N41" s="3" t="n"/>
       <c r="O41" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="P41" s="3" t="n">
-        <v>2</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="P41" s="3" t="n"/>
       <c r="Q41" s="3" t="n"/>
       <c r="R41" s="3" t="n"/>
       <c r="S41" s="3" t="n"/>
       <c r="T41" s="3" t="n"/>
       <c r="U41" s="3" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>2502HX</t>
-        </is>
-      </c>
-      <c r="B42" s="3" t="n">
-        <v>8</v>
-      </c>
+          <t>2502</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n"/>
       <c r="C42" s="3" t="n"/>
       <c r="D42" s="3" t="n"/>
       <c r="E42" s="3" t="n"/>
@@ -2959,24 +2901,28 @@
       <c r="L42" s="3" t="n"/>
       <c r="M42" s="3" t="n"/>
       <c r="N42" s="3" t="n"/>
-      <c r="O42" s="3" t="n"/>
-      <c r="P42" s="3" t="n"/>
+      <c r="O42" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="P42" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="Q42" s="3" t="n"/>
       <c r="R42" s="3" t="n"/>
       <c r="S42" s="3" t="n"/>
       <c r="T42" s="3" t="n"/>
       <c r="U42" s="3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>2503</t>
+          <t>2502HX</t>
         </is>
       </c>
       <c r="B43" s="3" t="n">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="C43" s="3" t="n"/>
       <c r="D43" s="3" t="n"/>
@@ -2997,17 +2943,17 @@
       <c r="S43" s="3" t="n"/>
       <c r="T43" s="3" t="n"/>
       <c r="U43" s="3" t="n">
-        <v>29</v>
+        <v>8</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>2504</t>
+          <t>2503</t>
         </is>
       </c>
       <c r="B44" s="3" t="n">
-        <v>4</v>
+        <v>29</v>
       </c>
       <c r="C44" s="3" t="n"/>
       <c r="D44" s="3" t="n"/>
@@ -3028,17 +2974,17 @@
       <c r="S44" s="3" t="n"/>
       <c r="T44" s="3" t="n"/>
       <c r="U44" s="3" t="n">
-        <v>4</v>
+        <v>29</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>2505</t>
+          <t>2504</t>
         </is>
       </c>
       <c r="B45" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C45" s="3" t="n"/>
       <c r="D45" s="3" t="n"/>
@@ -3050,9 +2996,7 @@
       <c r="J45" s="3" t="n"/>
       <c r="K45" s="3" t="n"/>
       <c r="L45" s="3" t="n"/>
-      <c r="M45" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="M45" s="3" t="n"/>
       <c r="N45" s="3" t="n"/>
       <c r="O45" s="3" t="n"/>
       <c r="P45" s="3" t="n"/>
@@ -3061,17 +3005,17 @@
       <c r="S45" s="3" t="n"/>
       <c r="T45" s="3" t="n"/>
       <c r="U45" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>2601</t>
+          <t>2505</t>
         </is>
       </c>
       <c r="B46" s="3" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C46" s="3" t="n"/>
       <c r="D46" s="3" t="n"/>
@@ -3083,7 +3027,9 @@
       <c r="J46" s="3" t="n"/>
       <c r="K46" s="3" t="n"/>
       <c r="L46" s="3" t="n"/>
-      <c r="M46" s="3" t="n"/>
+      <c r="M46" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="N46" s="3" t="n"/>
       <c r="O46" s="3" t="n"/>
       <c r="P46" s="3" t="n"/>
@@ -3092,17 +3038,17 @@
       <c r="S46" s="3" t="n"/>
       <c r="T46" s="3" t="n"/>
       <c r="U46" s="3" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>2602</t>
+          <t>2601</t>
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C47" s="3" t="n"/>
       <c r="D47" s="3" t="n"/>
@@ -3123,16 +3069,18 @@
       <c r="S47" s="3" t="n"/>
       <c r="T47" s="3" t="n"/>
       <c r="U47" s="3" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>2603</t>
-        </is>
-      </c>
-      <c r="B48" s="3" t="n"/>
+          <t>2602</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>6</v>
+      </c>
       <c r="C48" s="3" t="n"/>
       <c r="D48" s="3" t="n"/>
       <c r="E48" s="3" t="n"/>
@@ -3146,26 +3094,22 @@
       <c r="M48" s="3" t="n"/>
       <c r="N48" s="3" t="n"/>
       <c r="O48" s="3" t="n"/>
-      <c r="P48" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="P48" s="3" t="n"/>
       <c r="Q48" s="3" t="n"/>
       <c r="R48" s="3" t="n"/>
       <c r="S48" s="3" t="n"/>
       <c r="T48" s="3" t="n"/>
       <c r="U48" s="3" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>2603HX</t>
-        </is>
-      </c>
-      <c r="B49" s="3" t="n">
-        <v>11</v>
-      </c>
+          <t>2603</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n"/>
       <c r="C49" s="3" t="n"/>
       <c r="D49" s="3" t="n"/>
       <c r="E49" s="3" t="n"/>
@@ -3179,23 +3123,25 @@
       <c r="M49" s="3" t="n"/>
       <c r="N49" s="3" t="n"/>
       <c r="O49" s="3" t="n"/>
-      <c r="P49" s="3" t="n"/>
+      <c r="P49" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="Q49" s="3" t="n"/>
       <c r="R49" s="3" t="n"/>
       <c r="S49" s="3" t="n"/>
       <c r="T49" s="3" t="n"/>
       <c r="U49" s="3" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>2605</t>
+          <t>2603HX</t>
         </is>
       </c>
       <c r="B50" s="3" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C50" s="3" t="n"/>
       <c r="D50" s="3" t="n"/>
@@ -3216,17 +3162,17 @@
       <c r="S50" s="3" t="n"/>
       <c r="T50" s="3" t="n"/>
       <c r="U50" s="3" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>2606</t>
+          <t>2605</t>
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C51" s="3" t="n"/>
       <c r="D51" s="3" t="n"/>
@@ -3247,17 +3193,17 @@
       <c r="S51" s="3" t="n"/>
       <c r="T51" s="3" t="n"/>
       <c r="U51" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>2609</t>
+          <t>2606</t>
         </is>
       </c>
       <c r="B52" s="3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C52" s="3" t="n"/>
       <c r="D52" s="3" t="n"/>
@@ -3278,17 +3224,17 @@
       <c r="S52" s="3" t="n"/>
       <c r="T52" s="3" t="n"/>
       <c r="U52" s="3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>2611</t>
+          <t>2609</t>
         </is>
       </c>
       <c r="B53" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C53" s="3" t="n"/>
       <c r="D53" s="3" t="n"/>
@@ -3309,17 +3255,17 @@
       <c r="S53" s="3" t="n"/>
       <c r="T53" s="3" t="n"/>
       <c r="U53" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>2650</t>
+          <t>2611</t>
         </is>
       </c>
       <c r="B54" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C54" s="3" t="n"/>
       <c r="D54" s="3" t="n"/>
@@ -3340,17 +3286,17 @@
       <c r="S54" s="3" t="n"/>
       <c r="T54" s="3" t="n"/>
       <c r="U54" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>2650</t>
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="C55" s="3" t="n"/>
       <c r="D55" s="3" t="n"/>
@@ -3365,25 +3311,23 @@
       <c r="M55" s="3" t="n"/>
       <c r="N55" s="3" t="n"/>
       <c r="O55" s="3" t="n"/>
-      <c r="P55" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="P55" s="3" t="n"/>
       <c r="Q55" s="3" t="n"/>
       <c r="R55" s="3" t="n"/>
       <c r="S55" s="3" t="n"/>
       <c r="T55" s="3" t="n"/>
       <c r="U55" s="3" t="n">
-        <v>34</v>
+        <v>4</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>2701</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="B56" s="3" t="n">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="C56" s="3" t="n"/>
       <c r="D56" s="3" t="n"/>
@@ -3398,23 +3342,25 @@
       <c r="M56" s="3" t="n"/>
       <c r="N56" s="3" t="n"/>
       <c r="O56" s="3" t="n"/>
-      <c r="P56" s="3" t="n"/>
+      <c r="P56" s="3" t="n">
+        <v>8</v>
+      </c>
       <c r="Q56" s="3" t="n"/>
       <c r="R56" s="3" t="n"/>
       <c r="S56" s="3" t="n"/>
       <c r="T56" s="3" t="n"/>
       <c r="U56" s="3" t="n">
-        <v>15</v>
+        <v>34</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>2702</t>
+          <t>2701</t>
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C57" s="3" t="n"/>
       <c r="D57" s="3" t="n"/>
@@ -3427,9 +3373,7 @@
       <c r="K57" s="3" t="n"/>
       <c r="L57" s="3" t="n"/>
       <c r="M57" s="3" t="n"/>
-      <c r="N57" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="N57" s="3" t="n"/>
       <c r="O57" s="3" t="n"/>
       <c r="P57" s="3" t="n"/>
       <c r="Q57" s="3" t="n"/>
@@ -3437,17 +3381,17 @@
       <c r="S57" s="3" t="n"/>
       <c r="T57" s="3" t="n"/>
       <c r="U57" s="3" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>2703</t>
+          <t>2702</t>
         </is>
       </c>
       <c r="B58" s="3" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C58" s="3" t="n"/>
       <c r="D58" s="3" t="n"/>
@@ -3460,7 +3404,9 @@
       <c r="K58" s="3" t="n"/>
       <c r="L58" s="3" t="n"/>
       <c r="M58" s="3" t="n"/>
-      <c r="N58" s="3" t="n"/>
+      <c r="N58" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="O58" s="3" t="n"/>
       <c r="P58" s="3" t="n"/>
       <c r="Q58" s="3" t="n"/>
@@ -3474,7 +3420,7 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>2704</t>
+          <t>2703</t>
         </is>
       </c>
       <c r="B59" s="3" t="n">
@@ -3505,11 +3451,11 @@
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>2705</t>
+          <t>2704</t>
         </is>
       </c>
       <c r="B60" s="3" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C60" s="3" t="n"/>
       <c r="D60" s="3" t="n"/>
@@ -3524,25 +3470,23 @@
       <c r="M60" s="3" t="n"/>
       <c r="N60" s="3" t="n"/>
       <c r="O60" s="3" t="n"/>
-      <c r="P60" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="P60" s="3" t="n"/>
       <c r="Q60" s="3" t="n"/>
       <c r="R60" s="3" t="n"/>
       <c r="S60" s="3" t="n"/>
       <c r="T60" s="3" t="n"/>
       <c r="U60" s="3" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>2706</t>
+          <t>2705</t>
         </is>
       </c>
       <c r="B61" s="3" t="n">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="C61" s="3" t="n"/>
       <c r="D61" s="3" t="n"/>
@@ -3558,23 +3502,25 @@
       <c r="N61" s="3" t="n"/>
       <c r="O61" s="3" t="n"/>
       <c r="P61" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q61" s="3" t="n"/>
       <c r="R61" s="3" t="n"/>
       <c r="S61" s="3" t="n"/>
       <c r="T61" s="3" t="n"/>
       <c r="U61" s="3" t="n">
-        <v>29</v>
+        <v>17</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>3051</t>
-        </is>
-      </c>
-      <c r="B62" s="3" t="n"/>
+          <t>2706</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="n">
+        <v>25</v>
+      </c>
       <c r="C62" s="3" t="n"/>
       <c r="D62" s="3" t="n"/>
       <c r="E62" s="3" t="n"/>
@@ -3585,24 +3531,24 @@
       <c r="J62" s="3" t="n"/>
       <c r="K62" s="3" t="n"/>
       <c r="L62" s="3" t="n"/>
-      <c r="M62" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="M62" s="3" t="n"/>
       <c r="N62" s="3" t="n"/>
       <c r="O62" s="3" t="n"/>
-      <c r="P62" s="3" t="n"/>
+      <c r="P62" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="Q62" s="3" t="n"/>
       <c r="R62" s="3" t="n"/>
       <c r="S62" s="3" t="n"/>
       <c r="T62" s="3" t="n"/>
       <c r="U62" s="3" t="n">
-        <v>4</v>
+        <v>29</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>3474</t>
+          <t>3051</t>
         </is>
       </c>
       <c r="B63" s="3" t="n"/>
@@ -3616,24 +3562,24 @@
       <c r="J63" s="3" t="n"/>
       <c r="K63" s="3" t="n"/>
       <c r="L63" s="3" t="n"/>
-      <c r="M63" s="3" t="n"/>
+      <c r="M63" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="N63" s="3" t="n"/>
       <c r="O63" s="3" t="n"/>
       <c r="P63" s="3" t="n"/>
-      <c r="Q63" s="3" t="n">
-        <v>7</v>
-      </c>
+      <c r="Q63" s="3" t="n"/>
       <c r="R63" s="3" t="n"/>
       <c r="S63" s="3" t="n"/>
       <c r="T63" s="3" t="n"/>
       <c r="U63" s="3" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>4000</t>
+          <t>3474</t>
         </is>
       </c>
       <c r="B64" s="3" t="n"/>
@@ -3652,22 +3598,24 @@
       <c r="O64" s="3" t="n"/>
       <c r="P64" s="3" t="n"/>
       <c r="Q64" s="3" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="R64" s="3" t="n"/>
       <c r="S64" s="3" t="n"/>
       <c r="T64" s="3" t="n"/>
       <c r="U64" s="3" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>4001</t>
-        </is>
-      </c>
-      <c r="B65" s="3" t="n"/>
+          <t>4000</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="n">
+        <v>21</v>
+      </c>
       <c r="C65" s="3" t="n"/>
       <c r="D65" s="3" t="n"/>
       <c r="E65" s="3" t="n"/>
@@ -3682,14 +3630,12 @@
       <c r="N65" s="3" t="n"/>
       <c r="O65" s="3" t="n"/>
       <c r="P65" s="3" t="n"/>
-      <c r="Q65" s="3" t="n">
-        <v>10</v>
-      </c>
+      <c r="Q65" s="3" t="n"/>
       <c r="R65" s="3" t="n"/>
       <c r="S65" s="3" t="n"/>
       <c r="T65" s="3" t="n"/>
       <c r="U65" s="3" t="n">
-        <v>10</v>
+        <v>21</v>
       </c>
     </row>
     <row r="66">
@@ -3791,7 +3737,9 @@
           <t>4503</t>
         </is>
       </c>
-      <c r="B69" s="3" t="n"/>
+      <c r="B69" s="3" t="n">
+        <v>7</v>
+      </c>
       <c r="C69" s="3" t="n"/>
       <c r="D69" s="3" t="n"/>
       <c r="E69" s="3" t="n"/>
@@ -3802,9 +3750,7 @@
       <c r="J69" s="3" t="n"/>
       <c r="K69" s="3" t="n"/>
       <c r="L69" s="3" t="n"/>
-      <c r="M69" s="3" t="n">
-        <v>7</v>
-      </c>
+      <c r="M69" s="3" t="n"/>
       <c r="N69" s="3" t="n"/>
       <c r="O69" s="3" t="n"/>
       <c r="P69" s="3" t="n"/>
@@ -3853,7 +3799,9 @@
           <t>4603</t>
         </is>
       </c>
-      <c r="B71" s="3" t="n"/>
+      <c r="B71" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="C71" s="3" t="n"/>
       <c r="D71" s="3" t="n"/>
       <c r="E71" s="3" t="n"/>
@@ -3863,9 +3811,7 @@
       <c r="I71" s="3" t="n"/>
       <c r="J71" s="3" t="n"/>
       <c r="K71" s="3" t="n"/>
-      <c r="L71" s="3" t="n">
-        <v>5</v>
-      </c>
+      <c r="L71" s="3" t="n"/>
       <c r="M71" s="3" t="n"/>
       <c r="N71" s="3" t="n"/>
       <c r="O71" s="3" t="n"/>
@@ -12434,15 +12380,19 @@
       </c>
       <c r="E175" s="3" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F175" s="3" t="inlineStr">
         <is>
-          <t>Missing - Air-Way lists only the non-forged part (OMi sells -FG)</t>
-        </is>
-      </c>
-      <c r="G175" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G175" s="3" t="inlineStr">
+        <is>
+          <t>master 1603</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="3" t="inlineStr">
@@ -12721,22 +12671,22 @@
       </c>
       <c r="D183" s="3" t="inlineStr">
         <is>
-          <t>1700</t>
+          <t>1700RC</t>
         </is>
       </c>
       <c r="E183" s="3" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F183" s="3" t="inlineStr">
         <is>
-          <t>Needs one specific item (see note)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G183" s="3" t="inlineStr">
         <is>
-          <t>BUILD-MISSING: part exists in OMi catalog but Air-Way s-page has no row; needs a second di</t>
+          <t>master 1700RC</t>
         </is>
       </c>
     </row>
@@ -12832,22 +12782,22 @@
       </c>
       <c r="D186" s="3" t="inlineStr">
         <is>
-          <t>1700</t>
+          <t>1700RC</t>
         </is>
       </c>
       <c r="E186" s="3" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F186" s="3" t="inlineStr">
         <is>
-          <t>Needs one specific item (see note)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G186" s="3" t="inlineStr">
         <is>
-          <t>BUILD-MISSING: part exists in OMi catalog but Air-Way s-page has no row; needs a second di</t>
+          <t>master 1700RC</t>
         </is>
       </c>
     </row>
@@ -12943,22 +12893,22 @@
       </c>
       <c r="D189" s="3" t="inlineStr">
         <is>
-          <t>1700</t>
+          <t>1700RC</t>
         </is>
       </c>
       <c r="E189" s="3" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F189" s="3" t="inlineStr">
         <is>
-          <t>Needs one specific item (see note)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G189" s="3" t="inlineStr">
         <is>
-          <t>BUILD-MISSING: part exists in OMi catalog but Air-Way s-page has no row; needs a second di</t>
+          <t>master 1700RC</t>
         </is>
       </c>
     </row>
@@ -13484,17 +13434,17 @@
       </c>
       <c r="E205" s="3" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F205" s="3" t="inlineStr">
         <is>
-          <t>Needs one specific item (see note)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G205" s="3" t="inlineStr">
         <is>
-          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series (e.g. 1501 N</t>
+          <t>master 1703</t>
         </is>
       </c>
     </row>
@@ -14717,17 +14667,17 @@
       </c>
       <c r="E242" s="3" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F242" s="3" t="inlineStr">
         <is>
-          <t>Needs one specific item (see note)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G242" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">MISSING: needs a dimensional source (Air-Way sibling family, Parker/Brennan catalog, or a </t>
+          <t>master 1800</t>
         </is>
       </c>
     </row>
@@ -36145,15 +36095,19 @@
       </c>
       <c r="E838" s="3" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F838" s="3" t="inlineStr">
         <is>
-          <t>Missing - no Air-Way page for the whole series</t>
-        </is>
-      </c>
-      <c r="G838" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G838" s="3" t="inlineStr">
+        <is>
+          <t>master 4000</t>
+        </is>
+      </c>
     </row>
     <row r="839">
       <c r="A839" s="3" t="inlineStr">
@@ -36178,15 +36132,19 @@
       </c>
       <c r="E839" s="3" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F839" s="3" t="inlineStr">
         <is>
-          <t>Missing - no Air-Way page for the whole series</t>
-        </is>
-      </c>
-      <c r="G839" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G839" s="3" t="inlineStr">
+        <is>
+          <t>master 4000</t>
+        </is>
+      </c>
     </row>
     <row r="840">
       <c r="A840" s="3" t="inlineStr">
@@ -36211,15 +36169,19 @@
       </c>
       <c r="E840" s="3" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F840" s="3" t="inlineStr">
         <is>
-          <t>Missing - no Air-Way page for the whole series</t>
-        </is>
-      </c>
-      <c r="G840" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G840" s="3" t="inlineStr">
+        <is>
+          <t>master 4000</t>
+        </is>
+      </c>
     </row>
     <row r="841">
       <c r="A841" s="3" t="inlineStr">
@@ -36244,15 +36206,19 @@
       </c>
       <c r="E841" s="3" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F841" s="3" t="inlineStr">
         <is>
-          <t>Missing - no Air-Way page for the whole series</t>
-        </is>
-      </c>
-      <c r="G841" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G841" s="3" t="inlineStr">
+        <is>
+          <t>master 4000</t>
+        </is>
+      </c>
     </row>
     <row r="842">
       <c r="A842" s="3" t="inlineStr">
@@ -36277,15 +36243,19 @@
       </c>
       <c r="E842" s="3" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F842" s="3" t="inlineStr">
         <is>
-          <t>Missing - no Air-Way page for the whole series</t>
-        </is>
-      </c>
-      <c r="G842" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G842" s="3" t="inlineStr">
+        <is>
+          <t>master 4000</t>
+        </is>
+      </c>
     </row>
     <row r="843">
       <c r="A843" s="3" t="inlineStr">
@@ -36310,15 +36280,19 @@
       </c>
       <c r="E843" s="3" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F843" s="3" t="inlineStr">
         <is>
-          <t>Missing - no Air-Way page for the whole series</t>
-        </is>
-      </c>
-      <c r="G843" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G843" s="3" t="inlineStr">
+        <is>
+          <t>master 4000</t>
+        </is>
+      </c>
     </row>
     <row r="844">
       <c r="A844" s="3" t="inlineStr">
@@ -36343,15 +36317,19 @@
       </c>
       <c r="E844" s="3" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F844" s="3" t="inlineStr">
         <is>
-          <t>Missing - no Air-Way page for the whole series</t>
-        </is>
-      </c>
-      <c r="G844" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G844" s="3" t="inlineStr">
+        <is>
+          <t>master 4000</t>
+        </is>
+      </c>
     </row>
     <row r="845">
       <c r="A845" s="3" t="inlineStr">
@@ -36376,15 +36354,19 @@
       </c>
       <c r="E845" s="3" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F845" s="3" t="inlineStr">
         <is>
-          <t>Missing - no Air-Way page for the whole series</t>
-        </is>
-      </c>
-      <c r="G845" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G845" s="3" t="inlineStr">
+        <is>
+          <t>master 4000</t>
+        </is>
+      </c>
     </row>
     <row r="846">
       <c r="A846" s="3" t="inlineStr">
@@ -36409,15 +36391,19 @@
       </c>
       <c r="E846" s="3" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F846" s="3" t="inlineStr">
         <is>
-          <t>Missing - no Air-Way page for the whole series</t>
-        </is>
-      </c>
-      <c r="G846" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G846" s="3" t="inlineStr">
+        <is>
+          <t>master 4000</t>
+        </is>
+      </c>
     </row>
     <row r="847">
       <c r="A847" s="3" t="inlineStr">
@@ -36442,15 +36428,19 @@
       </c>
       <c r="E847" s="3" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F847" s="3" t="inlineStr">
         <is>
-          <t>Missing - no Air-Way page for the whole series</t>
-        </is>
-      </c>
-      <c r="G847" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G847" s="3" t="inlineStr">
+        <is>
+          <t>master 4000</t>
+        </is>
+      </c>
     </row>
     <row r="848">
       <c r="A848" s="3" t="inlineStr">
@@ -36475,15 +36465,19 @@
       </c>
       <c r="E848" s="3" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F848" s="3" t="inlineStr">
         <is>
-          <t>Missing - no Air-Way page for the whole series</t>
-        </is>
-      </c>
-      <c r="G848" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G848" s="3" t="inlineStr">
+        <is>
+          <t>master 4000</t>
+        </is>
+      </c>
     </row>
     <row r="849">
       <c r="A849" s="3" t="inlineStr">
@@ -36503,20 +36497,24 @@
       </c>
       <c r="D849" s="3" t="inlineStr">
         <is>
-          <t>4001</t>
+          <t>4000</t>
         </is>
       </c>
       <c r="E849" s="3" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F849" s="3" t="inlineStr">
         <is>
-          <t>Missing - no Air-Way page for the whole series</t>
-        </is>
-      </c>
-      <c r="G849" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G849" s="3" t="inlineStr">
+        <is>
+          <t>master 4000</t>
+        </is>
+      </c>
     </row>
     <row r="850">
       <c r="A850" s="3" t="inlineStr">
@@ -36536,20 +36534,24 @@
       </c>
       <c r="D850" s="3" t="inlineStr">
         <is>
-          <t>4001</t>
+          <t>4000</t>
         </is>
       </c>
       <c r="E850" s="3" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F850" s="3" t="inlineStr">
         <is>
-          <t>Missing - no Air-Way page for the whole series</t>
-        </is>
-      </c>
-      <c r="G850" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G850" s="3" t="inlineStr">
+        <is>
+          <t>master 4000</t>
+        </is>
+      </c>
     </row>
     <row r="851">
       <c r="A851" s="3" t="inlineStr">
@@ -36569,20 +36571,24 @@
       </c>
       <c r="D851" s="3" t="inlineStr">
         <is>
-          <t>4001</t>
+          <t>4000</t>
         </is>
       </c>
       <c r="E851" s="3" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F851" s="3" t="inlineStr">
         <is>
-          <t>Missing - no Air-Way page for the whole series</t>
-        </is>
-      </c>
-      <c r="G851" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G851" s="3" t="inlineStr">
+        <is>
+          <t>master 4000</t>
+        </is>
+      </c>
     </row>
     <row r="852">
       <c r="A852" s="3" t="inlineStr">
@@ -36602,20 +36608,24 @@
       </c>
       <c r="D852" s="3" t="inlineStr">
         <is>
-          <t>4001</t>
+          <t>4000</t>
         </is>
       </c>
       <c r="E852" s="3" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F852" s="3" t="inlineStr">
         <is>
-          <t>Missing - no Air-Way page for the whole series</t>
-        </is>
-      </c>
-      <c r="G852" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G852" s="3" t="inlineStr">
+        <is>
+          <t>master 4000</t>
+        </is>
+      </c>
     </row>
     <row r="853">
       <c r="A853" s="3" t="inlineStr">
@@ -36635,20 +36645,24 @@
       </c>
       <c r="D853" s="3" t="inlineStr">
         <is>
-          <t>4001</t>
+          <t>4000</t>
         </is>
       </c>
       <c r="E853" s="3" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F853" s="3" t="inlineStr">
         <is>
-          <t>Missing - no Air-Way page for the whole series</t>
-        </is>
-      </c>
-      <c r="G853" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G853" s="3" t="inlineStr">
+        <is>
+          <t>master 4000</t>
+        </is>
+      </c>
     </row>
     <row r="854">
       <c r="A854" s="3" t="inlineStr">
@@ -36668,20 +36682,24 @@
       </c>
       <c r="D854" s="3" t="inlineStr">
         <is>
-          <t>4001</t>
+          <t>4000</t>
         </is>
       </c>
       <c r="E854" s="3" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F854" s="3" t="inlineStr">
         <is>
-          <t>Missing - no Air-Way page for the whole series</t>
-        </is>
-      </c>
-      <c r="G854" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G854" s="3" t="inlineStr">
+        <is>
+          <t>master 4000</t>
+        </is>
+      </c>
     </row>
     <row r="855">
       <c r="A855" s="3" t="inlineStr">
@@ -36701,20 +36719,24 @@
       </c>
       <c r="D855" s="3" t="inlineStr">
         <is>
-          <t>4001</t>
+          <t>4000</t>
         </is>
       </c>
       <c r="E855" s="3" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F855" s="3" t="inlineStr">
         <is>
-          <t>Missing - no Air-Way page for the whole series</t>
-        </is>
-      </c>
-      <c r="G855" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G855" s="3" t="inlineStr">
+        <is>
+          <t>master 4000</t>
+        </is>
+      </c>
     </row>
     <row r="856">
       <c r="A856" s="3" t="inlineStr">
@@ -36734,20 +36756,24 @@
       </c>
       <c r="D856" s="3" t="inlineStr">
         <is>
-          <t>4001</t>
+          <t>4000</t>
         </is>
       </c>
       <c r="E856" s="3" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F856" s="3" t="inlineStr">
         <is>
-          <t>Missing - no Air-Way page for the whole series</t>
-        </is>
-      </c>
-      <c r="G856" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G856" s="3" t="inlineStr">
+        <is>
+          <t>master 4000</t>
+        </is>
+      </c>
     </row>
     <row r="857">
       <c r="A857" s="3" t="inlineStr">
@@ -36767,20 +36793,24 @@
       </c>
       <c r="D857" s="3" t="inlineStr">
         <is>
-          <t>4001</t>
+          <t>4000</t>
         </is>
       </c>
       <c r="E857" s="3" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F857" s="3" t="inlineStr">
         <is>
-          <t>Missing - no Air-Way page for the whole series</t>
-        </is>
-      </c>
-      <c r="G857" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G857" s="3" t="inlineStr">
+        <is>
+          <t>master 4000</t>
+        </is>
+      </c>
     </row>
     <row r="858">
       <c r="A858" s="3" t="inlineStr">
@@ -36800,20 +36830,24 @@
       </c>
       <c r="D858" s="3" t="inlineStr">
         <is>
-          <t>4001</t>
+          <t>4000</t>
         </is>
       </c>
       <c r="E858" s="3" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F858" s="3" t="inlineStr">
         <is>
-          <t>Missing - no Air-Way page for the whole series</t>
-        </is>
-      </c>
-      <c r="G858" s="3" t="inlineStr"/>
+          <t>Built - master in 11_MASTERS</t>
+        </is>
+      </c>
+      <c r="G858" s="3" t="inlineStr">
+        <is>
+          <t>master 4000</t>
+        </is>
+      </c>
     </row>
     <row r="859">
       <c r="A859" s="3" t="inlineStr">
@@ -38060,17 +38094,17 @@
       </c>
       <c r="E893" s="3" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F893" s="3" t="inlineStr">
         <is>
-          <t>Needs one specific item (see note)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G893" s="3" t="inlineStr">
         <is>
-          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series (e.g. 1501 N</t>
+          <t>master 4503</t>
         </is>
       </c>
     </row>
@@ -38097,17 +38131,17 @@
       </c>
       <c r="E894" s="3" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F894" s="3" t="inlineStr">
         <is>
-          <t>Needs one specific item (see note)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G894" s="3" t="inlineStr">
         <is>
-          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series (e.g. 1501 N</t>
+          <t>master 4503</t>
         </is>
       </c>
     </row>
@@ -38134,17 +38168,17 @@
       </c>
       <c r="E895" s="3" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F895" s="3" t="inlineStr">
         <is>
-          <t>Needs one specific item (see note)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G895" s="3" t="inlineStr">
         <is>
-          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series (e.g. 1501 N</t>
+          <t>master 4503</t>
         </is>
       </c>
     </row>
@@ -38171,17 +38205,17 @@
       </c>
       <c r="E896" s="3" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F896" s="3" t="inlineStr">
         <is>
-          <t>Needs one specific item (see note)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G896" s="3" t="inlineStr">
         <is>
-          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series (e.g. 1501 N</t>
+          <t>master 4503</t>
         </is>
       </c>
     </row>
@@ -38208,17 +38242,17 @@
       </c>
       <c r="E897" s="3" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F897" s="3" t="inlineStr">
         <is>
-          <t>Needs one specific item (see note)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G897" s="3" t="inlineStr">
         <is>
-          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series (e.g. 1501 N</t>
+          <t>master 4503</t>
         </is>
       </c>
     </row>
@@ -38245,17 +38279,17 @@
       </c>
       <c r="E898" s="3" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F898" s="3" t="inlineStr">
         <is>
-          <t>Needs one specific item (see note)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G898" s="3" t="inlineStr">
         <is>
-          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series (e.g. 1501 N</t>
+          <t>master 4503</t>
         </is>
       </c>
     </row>
@@ -38282,17 +38316,17 @@
       </c>
       <c r="E899" s="3" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F899" s="3" t="inlineStr">
         <is>
-          <t>Needs one specific item (see note)</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G899" s="3" t="inlineStr">
         <is>
-          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series (e.g. 1501 N</t>
+          <t>master 4503</t>
         </is>
       </c>
     </row>
@@ -38874,17 +38908,17 @@
       </c>
       <c r="E915" s="3" t="inlineStr">
         <is>
-          <t>D6</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F915" s="3" t="inlineStr">
         <is>
-          <t>Needs Brennan STEPs - adjustable ORB stud (nut/washer) sizes + a new module</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G915" s="3" t="inlineStr">
         <is>
-          <t>adjustable ORB stud + locknut + hose-barb leg</t>
+          <t>master 4603</t>
         </is>
       </c>
     </row>
@@ -38911,17 +38945,17 @@
       </c>
       <c r="E916" s="3" t="inlineStr">
         <is>
-          <t>D6</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F916" s="3" t="inlineStr">
         <is>
-          <t>Needs Brennan STEPs - adjustable ORB stud (nut/washer) sizes + a new module</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G916" s="3" t="inlineStr">
         <is>
-          <t>adjustable ORB stud + locknut + hose-barb leg</t>
+          <t>master 4603</t>
         </is>
       </c>
     </row>
@@ -38948,17 +38982,17 @@
       </c>
       <c r="E917" s="3" t="inlineStr">
         <is>
-          <t>D6</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F917" s="3" t="inlineStr">
         <is>
-          <t>Needs Brennan STEPs - adjustable ORB stud (nut/washer) sizes + a new module</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G917" s="3" t="inlineStr">
         <is>
-          <t>adjustable ORB stud + locknut + hose-barb leg</t>
+          <t>master 4603</t>
         </is>
       </c>
     </row>
@@ -38985,17 +39019,17 @@
       </c>
       <c r="E918" s="3" t="inlineStr">
         <is>
-          <t>D6</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F918" s="3" t="inlineStr">
         <is>
-          <t>Needs Brennan STEPs - adjustable ORB stud (nut/washer) sizes + a new module</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G918" s="3" t="inlineStr">
         <is>
-          <t>adjustable ORB stud + locknut + hose-barb leg</t>
+          <t>master 4603</t>
         </is>
       </c>
     </row>
@@ -39022,17 +39056,17 @@
       </c>
       <c r="E919" s="3" t="inlineStr">
         <is>
-          <t>D6</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F919" s="3" t="inlineStr">
         <is>
-          <t>Needs Brennan STEPs - adjustable ORB stud (nut/washer) sizes + a new module</t>
+          <t>Built - master in 11_MASTERS</t>
         </is>
       </c>
       <c r="G919" s="3" t="inlineStr">
         <is>
-          <t>adjustable ORB stud + locknut + hose-barb leg</t>
+          <t>master 4603</t>
         </is>
       </c>
     </row>

</xml_diff>